<commit_message>
Layout pelas fotos: esteiras lado a lado, transferência a cada 4 estações, alto giro atrás do operador
- transferência com rolete direcionador (2 estações à esquerda, 2 à direita; ponta 3/26)
- bacia volta à esteira de transporte de qualquer ponto da estação
- prateleiras alinhadas, caixa do endereço pelo tipo; 015 abre o lado direito do corredor
- 4 displays E+Q nos andares 4-5 (orçamento, documento e apresentação atualizados)
- bacia verde e operador com uniforme verde, calça e sapato pretos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TBWA3G7ku1j3oTf4VMkLud
</commit_message>
<xml_diff>
--- a/projeto/entregaveis/Orcamento_PTL.xlsx
+++ b/projeto/entregaveis/Orcamento_PTL.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Módulo Q — display de QUANTIDADE (3 dígitos) + botão com LED, um por endereço de alto giro (andares 0 a 3).</t>
   </si>
   <si>
-    <t xml:space="preserve">Módulo E+Q — display de ENDEREÇO (8 dígitos) + QUANTIDADE (3 dígitos) + botão; usado nos 2 blocos de alto giro dos andares 4-5 (esquerdo/direito) e em cada zona de baixo giro.</t>
+    <t xml:space="preserve">Módulo E+Q — display de ENDEREÇO (8 dígitos) + QUANTIDADE (3 dígitos) + botão; usado nos andares 4 e 5 do alto giro (1 por andar em cada lado: 4 por estação) e em cada zona de baixo giro.</t>
   </si>
   <si>
     <t xml:space="preserve">Nó de coluna — microcontrolador por coluna (prédio) do alto giro que liga os Módulos Q daquela coluna ao barramento RS-485.</t>
@@ -561,7 +561,7 @@
     <t xml:space="preserve">Coluna D (Piloto) = quantidade de estações nas linhas de total. Fonte: wms_endereco (cd_esteira 1 e 2), exportado em 23/10/2026; rua 90 (Marketing/Almoxarifado) desconsiderada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Regras: Alto giro = prédios 001-010; andares 4-5 viram 2 blocos E+Q (prédios 1-5 / 6-10). Baixo giro = demais prédios (fundo, 015 e esquinas), 1 zona E+Q a cada 4 prédios.</t>
+    <t xml:space="preserve">Regras: Alto giro = prédios 001-010; andares 4-5 com 4 displays E+Q por estação (A4 e A5 nos lados 001-005 e 006-010). Baixo giro = demais prédios (corredor, 015 e esquinas), 1 zona E+Q a cada 4 prédios.</t>
   </si>
   <si>
     <t xml:space="preserve">Código</t>
@@ -2404,15 +2404,15 @@
       </c>
       <c r="C4" s="10" t="n">
         <f aca="false">'A-Interno'!F13</f>
-        <v>10443.4012151639</v>
+        <v>10993.9714446721</v>
       </c>
       <c r="D4" s="10" t="n">
         <f aca="false">'A-Interno'!G13</f>
-        <v>187235.880303279</v>
+        <v>199238.884893443</v>
       </c>
       <c r="E4" s="11" t="n">
         <f aca="false">D4/Estações!$O$43</f>
-        <v>4680.89700758197</v>
+        <v>4980.97212233607</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2424,15 +2424,15 @@
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">'A-Interno'!F30</f>
-        <v>10354.4612151639</v>
+        <v>10873.0314446721</v>
       </c>
       <c r="D5" s="10" t="n">
         <f aca="false">'A-Interno'!G30</f>
-        <v>185656.760303279</v>
+        <v>196955.764893443</v>
       </c>
       <c r="E5" s="11" t="n">
         <f aca="false">D5/Estações!$O$43</f>
-        <v>4641.41900758197</v>
+        <v>4923.89412233607</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2444,15 +2444,15 @@
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">'A-Interno'!F24</f>
-        <v>13875.3279636302</v>
+        <v>14565.6204017273</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">'A-Interno'!G24</f>
-        <v>254686.776499598</v>
+        <v>269763.669678719</v>
       </c>
       <c r="E6" s="11" t="n">
         <f aca="false">D6/Estações!$O$43</f>
-        <v>6367.16941248994</v>
+        <v>6744.09174196797</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2464,15 +2464,15 @@
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">'A-Terceiros'!F10</f>
-        <v>31822.4277219551</v>
+        <v>32808.1033114633</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">'A-Terceiros'!G10</f>
-        <v>326284.963278119</v>
+        <v>347860.285788283</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">D7/Estações!$O$43</f>
-        <v>8157.12408195298</v>
+        <v>8696.50714470708</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2484,15 +2484,15 @@
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">'A-Terceiros'!F20</f>
-        <v>40650.4697219551</v>
+        <v>43195.6421514633</v>
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">'A-Terceiros'!G20</f>
-        <v>796445.526248119</v>
+        <v>852329.779238283</v>
       </c>
       <c r="E8" s="11" t="n">
         <f aca="false">D8/Estações!$O$43</f>
-        <v>19911.138156203</v>
+        <v>21308.2444809571</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2504,15 +2504,15 @@
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">'B-RFID'!F10</f>
-        <v>15205.4074319329</v>
+        <v>15895.69987003</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">'B-RFID'!G10</f>
-        <v>279129.135927001</v>
+        <v>294206.029106122</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">D9/Estações!$O$43</f>
-        <v>6978.22839817501</v>
+        <v>7355.15072765304</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2524,15 +2524,15 @@
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">'B-RFID'!F15</f>
-        <v>15048.1306804494</v>
+        <v>15738.4231185465</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">'B-RFID'!G15</f>
-        <v>278142.830835982</v>
+        <v>293219.724015103</v>
       </c>
       <c r="E10" s="11" t="n">
         <f aca="false">D10/Estações!$O$43</f>
-        <v>6953.57077089954</v>
+        <v>7330.49310037757</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3039,7 +3039,7 @@
         <v>20</v>
       </c>
       <c r="H2" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I2" s="21" t="n">
         <v>82</v>
@@ -3055,11 +3055,11 @@
       </c>
       <c r="M2" s="22" t="n">
         <f aca="false">H2+J2</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N2" s="22" t="n">
         <f aca="false">K2+M2+2</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O2" s="21" t="n">
         <v>1</v>
@@ -3088,7 +3088,7 @@
         <v>16</v>
       </c>
       <c r="H3" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>156</v>
@@ -3104,11 +3104,11 @@
       </c>
       <c r="M3" s="22" t="n">
         <f aca="false">H3+J3</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N3" s="22" t="n">
         <f aca="false">K3+M3+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O3" s="21" t="n">
         <v>1</v>
@@ -3137,7 +3137,7 @@
         <v>20</v>
       </c>
       <c r="H4" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I4" s="21" t="n">
         <v>160</v>
@@ -3153,11 +3153,11 @@
       </c>
       <c r="M4" s="22" t="n">
         <f aca="false">H4+J4</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N4" s="22" t="n">
         <f aca="false">K4+M4+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O4" s="21" t="n">
         <v>1</v>
@@ -3186,7 +3186,7 @@
         <v>20</v>
       </c>
       <c r="H5" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I5" s="21" t="n">
         <v>160</v>
@@ -3202,11 +3202,11 @@
       </c>
       <c r="M5" s="22" t="n">
         <f aca="false">H5+J5</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N5" s="22" t="n">
         <f aca="false">K5+M5+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>1</v>
@@ -3235,7 +3235,7 @@
         <v>20</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I6" s="21" t="n">
         <v>160</v>
@@ -3251,11 +3251,11 @@
       </c>
       <c r="M6" s="22" t="n">
         <f aca="false">H6+J6</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N6" s="22" t="n">
         <f aca="false">K6+M6+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>1</v>
@@ -3284,7 +3284,7 @@
         <v>16</v>
       </c>
       <c r="H7" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I7" s="21" t="n">
         <v>160</v>
@@ -3300,11 +3300,11 @@
       </c>
       <c r="M7" s="22" t="n">
         <f aca="false">H7+J7</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N7" s="22" t="n">
         <f aca="false">K7+M7+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>1</v>
@@ -3333,7 +3333,7 @@
         <v>20</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I8" s="21" t="n">
         <v>192</v>
@@ -3349,11 +3349,11 @@
       </c>
       <c r="M8" s="22" t="n">
         <f aca="false">H8+J8</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N8" s="22" t="n">
         <f aca="false">K8+M8+2</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>1</v>
@@ -3382,7 +3382,7 @@
         <v>20</v>
       </c>
       <c r="H9" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I9" s="21" t="n">
         <v>188</v>
@@ -3398,11 +3398,11 @@
       </c>
       <c r="M9" s="22" t="n">
         <f aca="false">H9+J9</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N9" s="22" t="n">
         <f aca="false">K9+M9+2</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         <v>16</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I10" s="21" t="n">
         <v>160</v>
@@ -3447,11 +3447,11 @@
       </c>
       <c r="M10" s="22" t="n">
         <f aca="false">H10+J10</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N10" s="22" t="n">
         <f aca="false">K10+M10+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>1</v>
@@ -3480,7 +3480,7 @@
         <v>20</v>
       </c>
       <c r="H11" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I11" s="21" t="n">
         <v>160</v>
@@ -3496,11 +3496,11 @@
       </c>
       <c r="M11" s="22" t="n">
         <f aca="false">H11+J11</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N11" s="22" t="n">
         <f aca="false">K11+M11+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>1</v>
@@ -3529,7 +3529,7 @@
         <v>14</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" s="21" t="n">
         <v>160</v>
@@ -3545,11 +3545,11 @@
       </c>
       <c r="M12" s="22" t="n">
         <f aca="false">H12+J12</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N12" s="22" t="n">
         <f aca="false">K12+M12+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1</v>
@@ -3578,7 +3578,7 @@
         <v>20</v>
       </c>
       <c r="H13" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I13" s="21" t="n">
         <v>160</v>
@@ -3594,11 +3594,11 @@
       </c>
       <c r="M13" s="22" t="n">
         <f aca="false">H13+J13</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N13" s="22" t="n">
         <f aca="false">K13+M13+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1</v>
@@ -3627,7 +3627,7 @@
         <v>10</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I14" s="21" t="n">
         <v>192</v>
@@ -3643,11 +3643,11 @@
       </c>
       <c r="M14" s="22" t="n">
         <f aca="false">H14+J14</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N14" s="22" t="n">
         <f aca="false">K14+M14+2</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>1</v>
@@ -3676,7 +3676,7 @@
         <v>20</v>
       </c>
       <c r="H15" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I15" s="21" t="n">
         <v>188</v>
@@ -3692,11 +3692,11 @@
       </c>
       <c r="M15" s="22" t="n">
         <f aca="false">H15+J15</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N15" s="22" t="n">
         <f aca="false">K15+M15+2</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O15" s="21" t="n">
         <v>1</v>
@@ -3725,7 +3725,7 @@
         <v>16</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I16" s="21" t="n">
         <v>160</v>
@@ -3741,11 +3741,11 @@
       </c>
       <c r="M16" s="22" t="n">
         <f aca="false">H16+J16</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N16" s="22" t="n">
         <f aca="false">K16+M16+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O16" s="21" t="n">
         <v>1</v>
@@ -3774,7 +3774,7 @@
         <v>20</v>
       </c>
       <c r="H17" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" s="21" t="n">
         <v>160</v>
@@ -3790,11 +3790,11 @@
       </c>
       <c r="M17" s="22" t="n">
         <f aca="false">H17+J17</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N17" s="22" t="n">
         <f aca="false">K17+M17+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O17" s="21" t="n">
         <v>1</v>
@@ -3823,7 +3823,7 @@
         <v>14</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" s="21" t="n">
         <v>160</v>
@@ -3839,11 +3839,11 @@
       </c>
       <c r="M18" s="22" t="n">
         <f aca="false">H18+J18</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N18" s="22" t="n">
         <f aca="false">K18+M18+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O18" s="21" t="n">
         <v>1</v>
@@ -3872,7 +3872,7 @@
         <v>20</v>
       </c>
       <c r="H19" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19" s="21" t="n">
         <v>160</v>
@@ -3888,11 +3888,11 @@
       </c>
       <c r="M19" s="22" t="n">
         <f aca="false">H19+J19</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N19" s="22" t="n">
         <f aca="false">K19+M19+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O19" s="21" t="n">
         <v>1</v>
@@ -3921,7 +3921,7 @@
         <v>10</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20" s="21" t="n">
         <v>160</v>
@@ -3937,11 +3937,11 @@
       </c>
       <c r="M20" s="22" t="n">
         <f aca="false">H20+J20</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N20" s="22" t="n">
         <f aca="false">K20+M20+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O20" s="21" t="n">
         <v>1</v>
@@ -3970,7 +3970,7 @@
         <v>10</v>
       </c>
       <c r="H21" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I21" s="21" t="n">
         <v>4</v>
@@ -3986,11 +3986,11 @@
       </c>
       <c r="M21" s="22" t="n">
         <f aca="false">H21+J21</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N21" s="22" t="n">
         <f aca="false">K21+M21+2</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="O21" s="21" t="n">
         <v>1</v>
@@ -4019,7 +4019,7 @@
         <v>13</v>
       </c>
       <c r="H22" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I22" s="21" t="n">
         <v>128</v>
@@ -4035,11 +4035,11 @@
       </c>
       <c r="M22" s="22" t="n">
         <f aca="false">H22+J22</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N22" s="22" t="n">
         <f aca="false">K22+M22+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O22" s="21" t="n">
         <v>1</v>
@@ -4068,7 +4068,7 @@
         <v>15</v>
       </c>
       <c r="H23" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" s="21" t="n">
         <v>131</v>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="M23" s="22" t="n">
         <f aca="false">H23+J23</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N23" s="22" t="n">
         <f aca="false">K23+M23+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O23" s="21" t="n">
         <v>1</v>
@@ -4117,7 +4117,7 @@
         <v>15</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" s="21" t="n">
         <v>131</v>
@@ -4133,11 +4133,11 @@
       </c>
       <c r="M24" s="22" t="n">
         <f aca="false">H24+J24</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N24" s="22" t="n">
         <f aca="false">K24+M24+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O24" s="21" t="n">
         <v>1</v>
@@ -4166,7 +4166,7 @@
         <v>15</v>
       </c>
       <c r="H25" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I25" s="21" t="n">
         <v>131</v>
@@ -4182,11 +4182,11 @@
       </c>
       <c r="M25" s="22" t="n">
         <f aca="false">H25+J25</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N25" s="22" t="n">
         <f aca="false">K25+M25+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O25" s="21" t="n">
         <v>1</v>
@@ -4215,7 +4215,7 @@
         <v>13</v>
       </c>
       <c r="H26" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I26" s="21" t="n">
         <v>131</v>
@@ -4231,11 +4231,11 @@
       </c>
       <c r="M26" s="22" t="n">
         <f aca="false">H26+J26</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N26" s="22" t="n">
         <f aca="false">K26+M26+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O26" s="21" t="n">
         <v>1</v>
@@ -4264,7 +4264,7 @@
         <v>15</v>
       </c>
       <c r="H27" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I27" s="21" t="n">
         <v>131</v>
@@ -4280,11 +4280,11 @@
       </c>
       <c r="M27" s="22" t="n">
         <f aca="false">H27+J27</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N27" s="22" t="n">
         <f aca="false">K27+M27+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O27" s="21" t="n">
         <v>1</v>
@@ -4313,7 +4313,7 @@
         <v>15</v>
       </c>
       <c r="H28" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I28" s="21" t="n">
         <v>230</v>
@@ -4329,11 +4329,11 @@
       </c>
       <c r="M28" s="22" t="n">
         <f aca="false">H28+J28</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N28" s="22" t="n">
         <f aca="false">K28+M28+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O28" s="21" t="n">
         <v>1</v>
@@ -4362,7 +4362,7 @@
         <v>15</v>
       </c>
       <c r="H29" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I29" s="21" t="n">
         <v>227</v>
@@ -4378,11 +4378,11 @@
       </c>
       <c r="M29" s="22" t="n">
         <f aca="false">H29+J29</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N29" s="22" t="n">
         <f aca="false">K29+M29+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O29" s="21" t="n">
         <v>1</v>
@@ -4411,7 +4411,7 @@
         <v>13</v>
       </c>
       <c r="H30" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I30" s="21" t="n">
         <v>131</v>
@@ -4427,11 +4427,11 @@
       </c>
       <c r="M30" s="22" t="n">
         <f aca="false">H30+J30</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N30" s="22" t="n">
         <f aca="false">K30+M30+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O30" s="21" t="n">
         <v>1</v>
@@ -4460,7 +4460,7 @@
         <v>15</v>
       </c>
       <c r="H31" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I31" s="21" t="n">
         <v>131</v>
@@ -4476,11 +4476,11 @@
       </c>
       <c r="M31" s="22" t="n">
         <f aca="false">H31+J31</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N31" s="22" t="n">
         <f aca="false">K31+M31+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O31" s="21" t="n">
         <v>1</v>
@@ -4509,7 +4509,7 @@
         <v>11</v>
       </c>
       <c r="H32" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I32" s="21" t="n">
         <v>131</v>
@@ -4525,11 +4525,11 @@
       </c>
       <c r="M32" s="22" t="n">
         <f aca="false">H32+J32</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N32" s="22" t="n">
         <f aca="false">K32+M32+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O32" s="21" t="n">
         <v>1</v>
@@ -4558,7 +4558,7 @@
         <v>15</v>
       </c>
       <c r="H33" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I33" s="21" t="n">
         <v>131</v>
@@ -4574,11 +4574,11 @@
       </c>
       <c r="M33" s="22" t="n">
         <f aca="false">H33+J33</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N33" s="22" t="n">
         <f aca="false">K33+M33+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O33" s="21" t="n">
         <v>1</v>
@@ -4607,7 +4607,7 @@
         <v>9</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I34" s="21" t="n">
         <v>230</v>
@@ -4623,11 +4623,11 @@
       </c>
       <c r="M34" s="22" t="n">
         <f aca="false">H34+J34</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N34" s="22" t="n">
         <f aca="false">K34+M34+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O34" s="21" t="n">
         <v>1</v>
@@ -4656,7 +4656,7 @@
         <v>15</v>
       </c>
       <c r="H35" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I35" s="21" t="n">
         <v>227</v>
@@ -4672,11 +4672,11 @@
       </c>
       <c r="M35" s="22" t="n">
         <f aca="false">H35+J35</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N35" s="22" t="n">
         <f aca="false">K35+M35+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O35" s="21" t="n">
         <v>1</v>
@@ -4705,7 +4705,7 @@
         <v>13</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I36" s="21" t="n">
         <v>131</v>
@@ -4721,11 +4721,11 @@
       </c>
       <c r="M36" s="22" t="n">
         <f aca="false">H36+J36</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N36" s="22" t="n">
         <f aca="false">K36+M36+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O36" s="21" t="n">
         <v>1</v>
@@ -4754,7 +4754,7 @@
         <v>15</v>
       </c>
       <c r="H37" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I37" s="21" t="n">
         <v>131</v>
@@ -4770,11 +4770,11 @@
       </c>
       <c r="M37" s="22" t="n">
         <f aca="false">H37+J37</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N37" s="22" t="n">
         <f aca="false">K37+M37+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O37" s="21" t="n">
         <v>1</v>
@@ -4803,7 +4803,7 @@
         <v>11</v>
       </c>
       <c r="H38" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38" s="21" t="n">
         <v>131</v>
@@ -4819,11 +4819,11 @@
       </c>
       <c r="M38" s="22" t="n">
         <f aca="false">H38+J38</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N38" s="22" t="n">
         <f aca="false">K38+M38+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O38" s="21" t="n">
         <v>1</v>
@@ -4852,7 +4852,7 @@
         <v>15</v>
       </c>
       <c r="H39" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39" s="21" t="n">
         <v>131</v>
@@ -4868,11 +4868,11 @@
       </c>
       <c r="M39" s="22" t="n">
         <f aca="false">H39+J39</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N39" s="22" t="n">
         <f aca="false">K39+M39+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O39" s="21" t="n">
         <v>1</v>
@@ -4901,7 +4901,7 @@
         <v>7</v>
       </c>
       <c r="H40" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I40" s="21" t="n">
         <v>131</v>
@@ -4917,11 +4917,11 @@
       </c>
       <c r="M40" s="22" t="n">
         <f aca="false">H40+J40</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N40" s="22" t="n">
         <f aca="false">K40+M40+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O40" s="21" t="n">
         <v>1</v>
@@ -4950,7 +4950,7 @@
         <v>15</v>
       </c>
       <c r="H41" s="21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I41" s="21" t="n">
         <v>131</v>
@@ -4966,11 +4966,11 @@
       </c>
       <c r="M41" s="22" t="n">
         <f aca="false">H41+J41</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N41" s="22" t="n">
         <f aca="false">K41+M41+2</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O41" s="21" t="n">
         <v>1</v>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H43" s="25" t="n">
         <f aca="false">SUM(H2:H41)</f>
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="I43" s="25" t="n">
         <f aca="false">SUM(I2:I41)</f>
@@ -5018,11 +5018,11 @@
       </c>
       <c r="M43" s="25" t="n">
         <f aca="false">SUM(M2:M41)</f>
-        <v>328</v>
+        <v>408</v>
       </c>
       <c r="N43" s="25" t="n">
         <f aca="false">SUM(N2:N41)</f>
-        <v>808</v>
+        <v>888</v>
       </c>
       <c r="O43" s="25" t="n">
         <f aca="false">SUM(O2:O41)</f>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="H44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",H2:H41)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",I2:I41)</f>
@@ -5071,11 +5071,11 @@
       </c>
       <c r="M44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",M2:M41)</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",N2:N41)</f>
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="O44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",O2:O41)</f>
@@ -7285,11 +7285,11 @@
       </c>
       <c r="C5" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$14),0)</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D5" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$43*(1+Premissas!$B$14),0)</f>
-        <v>361</v>
+        <v>449</v>
       </c>
       <c r="E5" s="33" t="n">
         <f aca="false">Composição!$F$27</f>
@@ -7297,11 +7297,11 @@
       </c>
       <c r="F5" s="27" t="n">
         <f aca="false">C5*E5</f>
-        <v>2231.1</v>
+        <v>2726.9</v>
       </c>
       <c r="G5" s="27" t="n">
         <f aca="false">D5*E5</f>
-        <v>44745.95</v>
+        <v>55653.55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7341,11 +7341,11 @@
       </c>
       <c r="C7" s="37" t="n">
         <f aca="false">Estações!$N$44*Premissas!$B$15</f>
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="D7" s="37" t="n">
         <f aca="false">Estações!$N$43*Premissas!$B$15</f>
-        <v>2424</v>
+        <v>2664</v>
       </c>
       <c r="E7" s="33" t="n">
         <f aca="false">Preços!$D$13</f>
@@ -7353,11 +7353,11 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">C7*E7</f>
-        <v>483.702295081967</v>
+        <v>532.072524590164</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">D7*E7</f>
-        <v>9770.78636065574</v>
+        <v>10738.1909508197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7369,11 +7369,11 @@
       </c>
       <c r="C8" s="37" t="n">
         <f aca="false">Estações!$N$44*2</f>
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="D8" s="37" t="n">
         <f aca="false">Estações!$N$43*2</f>
-        <v>1616</v>
+        <v>1776</v>
       </c>
       <c r="E8" s="33" t="n">
         <f aca="false">Preços!$D$12</f>
@@ -7381,11 +7381,11 @@
       </c>
       <c r="F8" s="27" t="n">
         <f aca="false">C8*E8</f>
-        <v>64</v>
+        <v>70.4</v>
       </c>
       <c r="G8" s="27" t="n">
         <f aca="false">D8*E8</f>
-        <v>1292.8</v>
+        <v>1420.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7510,11 +7510,11 @@
       <c r="E13" s="35"/>
       <c r="F13" s="36" t="n">
         <f aca="false">SUM(F3:F12)</f>
-        <v>10443.4012151639</v>
+        <v>10993.9714446721</v>
       </c>
       <c r="G13" s="36" t="n">
         <f aca="false">SUM(G3:G12)</f>
-        <v>187235.880303279</v>
+        <v>199238.884893443</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7587,11 +7587,11 @@
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">C5*Premissas!$B$10</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">D5*Premissas!$B$10</f>
-        <v>361</v>
+        <v>449</v>
       </c>
       <c r="E18" s="33" t="n">
         <f aca="false">Premissas!$B$7</f>
@@ -7599,11 +7599,11 @@
       </c>
       <c r="F18" s="27" t="n">
         <f aca="false">C18*E18</f>
-        <v>628.749938650307</v>
+        <v>768.472147239264</v>
       </c>
       <c r="G18" s="27" t="n">
         <f aca="false">D18*E18</f>
-        <v>12609.9293251534</v>
+        <v>15683.8179141104</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7697,20 +7697,20 @@
       <c r="B22" s="35"/>
       <c r="C22" s="38" t="n">
         <f aca="false">SUM(C16:C21)</f>
-        <v>98.25</v>
+        <v>102.25</v>
       </c>
       <c r="D22" s="38" t="n">
         <f aca="false">SUM(D16:D21)</f>
-        <v>1931</v>
+        <v>2019</v>
       </c>
       <c r="E22" s="35"/>
       <c r="F22" s="36" t="n">
         <f aca="false">SUM(F16:F21)</f>
-        <v>3431.92674846626</v>
+        <v>3571.64895705522</v>
       </c>
       <c r="G22" s="36" t="n">
         <f aca="false">SUM(G16:G21)</f>
-        <v>67450.896196319</v>
+        <v>70524.7847852761</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7723,11 +7723,11 @@
       <c r="E24" s="35"/>
       <c r="F24" s="36" t="n">
         <f aca="false">F13+F22</f>
-        <v>13875.3279636302</v>
+        <v>14565.6204017273</v>
       </c>
       <c r="G24" s="36" t="n">
         <f aca="false">G13+G22</f>
-        <v>254686.776499598</v>
+        <v>269763.669678719</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7744,11 +7744,11 @@
       </c>
       <c r="C27" s="37" t="n">
         <f aca="false">-(C4+C5+C6)</f>
-        <v>-43</v>
+        <v>-47</v>
       </c>
       <c r="D27" s="37" t="n">
         <f aca="false">-(D4+D5+D6)</f>
-        <v>-845</v>
+        <v>-933</v>
       </c>
       <c r="E27" s="33" t="n">
         <f aca="false">Preços!$D$9</f>
@@ -7756,11 +7756,11 @@
       </c>
       <c r="F27" s="27" t="n">
         <f aca="false">C27*E27</f>
-        <v>-344</v>
+        <v>-376</v>
       </c>
       <c r="G27" s="27" t="n">
         <f aca="false">D27*E27</f>
-        <v>-6760</v>
+        <v>-7464</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7829,11 +7829,11 @@
       <c r="E30" s="35"/>
       <c r="F30" s="36" t="n">
         <f aca="false">F13+SUM(F27:F29)</f>
-        <v>10354.4612151639</v>
+        <v>10873.0314446721</v>
       </c>
       <c r="G30" s="36" t="n">
         <f aca="false">G13+SUM(G27:G29)</f>
-        <v>185656.760303279</v>
+        <v>196955.764893443</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7961,11 +7961,11 @@
       </c>
       <c r="C4" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$14),0)</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D4" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$43*(1+Premissas!$B$14),0)</f>
-        <v>361</v>
+        <v>449</v>
       </c>
       <c r="E4" s="33" t="n">
         <f aca="false">Preços!$D$34+Preços!$D$15+Preços!$D$10</f>
@@ -7973,11 +7973,11 @@
       </c>
       <c r="F4" s="27" t="n">
         <f aca="false">C4*E4</f>
-        <v>4189.07412</v>
+        <v>5119.97948</v>
       </c>
       <c r="G4" s="27" t="n">
         <f aca="false">D4*E4</f>
-        <v>84014.20874</v>
+        <v>104494.12666</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8017,11 +8017,11 @@
       </c>
       <c r="C6" s="37" t="n">
         <f aca="false">(Estações!$F$44+Estações!$M$44)*Premissas!$B$15</f>
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="D6" s="37" t="n">
         <f aca="false">(Estações!$F$43+Estações!$M$43)*Premissas!$B$15</f>
-        <v>4824</v>
+        <v>5064</v>
       </c>
       <c r="E6" s="33" t="n">
         <f aca="false">Preços!$D$13+2*Preços!$D$12/Premissas!$B$15</f>
@@ -8029,11 +8029,11 @@
       </c>
       <c r="F6" s="27" t="n">
         <f aca="false">C6*E6</f>
-        <v>1095.40459016393</v>
+        <v>1150.17481967213</v>
       </c>
       <c r="G6" s="27" t="n">
         <f aca="false">D6*E6</f>
-        <v>22017.6322622951</v>
+        <v>23113.036852459</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8123,11 +8123,11 @@
       <c r="E10" s="35"/>
       <c r="F10" s="36" t="n">
         <f aca="false">SUM(F3:F9)</f>
-        <v>31822.4277219551</v>
+        <v>32808.1033114633</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">SUM(G3:G9)</f>
-        <v>326284.963278119</v>
+        <v>347860.285788283</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8172,11 +8172,11 @@
       </c>
       <c r="C14" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$14),0)</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D14" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$43*(1+Premissas!$B$14),0)</f>
-        <v>361</v>
+        <v>449</v>
       </c>
       <c r="E14" s="33" t="n">
         <f aca="false">Preços!$D$31</f>
@@ -8184,11 +8184,11 @@
       </c>
       <c r="F14" s="27" t="n">
         <f aca="false">C14*E14</f>
-        <v>11206.8099</v>
+        <v>13697.2121</v>
       </c>
       <c r="G14" s="27" t="n">
         <f aca="false">D14*E14</f>
-        <v>224758.79855</v>
+        <v>279547.64695</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8256,11 +8256,11 @@
       </c>
       <c r="C17" s="37" t="n">
         <f aca="false">(Estações!$F$44+Estações!$M$44)*Premissas!$B$15</f>
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="D17" s="37" t="n">
         <f aca="false">(Estações!$F$43+Estações!$M$43)*Premissas!$B$15</f>
-        <v>4824</v>
+        <v>5064</v>
       </c>
       <c r="E17" s="33" t="n">
         <f aca="false">Preços!$D$13+2*Preços!$D$12/Premissas!$B$15</f>
@@ -8268,11 +8268,11 @@
       </c>
       <c r="F17" s="27" t="n">
         <f aca="false">C17*E17</f>
-        <v>1095.40459016393</v>
+        <v>1150.17481967213</v>
       </c>
       <c r="G17" s="27" t="n">
         <f aca="false">D17*E17</f>
-        <v>22017.6322622951</v>
+        <v>23113.036852459</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8336,11 +8336,11 @@
       <c r="E20" s="35"/>
       <c r="F20" s="36" t="n">
         <f aca="false">SUM(F13:F19)</f>
-        <v>40650.4697219551</v>
+        <v>43195.6421514633</v>
       </c>
       <c r="G20" s="36" t="n">
         <f aca="false">SUM(G13:G19)</f>
-        <v>796445.526248119</v>
+        <v>852329.779238283</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8416,11 +8416,11 @@
       <c r="E3" s="13"/>
       <c r="F3" s="33" t="n">
         <f aca="false">'A-Interno'!F24</f>
-        <v>13875.3279636302</v>
+        <v>14565.6204017273</v>
       </c>
       <c r="G3" s="33" t="n">
         <f aca="false">'A-Interno'!G24</f>
-        <v>254686.776499598</v>
+        <v>269763.669678719</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8550,11 +8550,11 @@
       <c r="E10" s="35"/>
       <c r="F10" s="36" t="n">
         <f aca="false">F3+F4+F5+F8+F9</f>
-        <v>15205.4074319329</v>
+        <v>15895.69987003</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">G3+G4+G5+G8+G9</f>
-        <v>279129.135927001</v>
+        <v>294206.029106122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8628,11 +8628,11 @@
       <c r="E15" s="35"/>
       <c r="F15" s="36" t="n">
         <f aca="false">F3+F4+F5+F13+F14</f>
-        <v>15048.1306804494</v>
+        <v>15738.4231185465</v>
       </c>
       <c r="G15" s="36" t="n">
         <f aca="false">G3+G4+G5+G13+G14</f>
-        <v>278142.830835982</v>
+        <v>293219.724015103</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Separação aberta na frente, 4 zonas por lado no baixo giro com displays na altura dos olhos
- esteira de transporte por dentro do alto giro; separação na frente, aberta
- baixo giro: 4 zonas por lado (E1-E4, D1-D4), display E+Q a ~1,5 m; profundidade ~2 m
- caixas de endereço menores
- orçamento, diagramas, documento e apresentação atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TBWA3G7ku1j3oTf4VMkLud
</commit_message>
<xml_diff>
--- a/projeto/entregaveis/Orcamento_PTL.xlsx
+++ b/projeto/entregaveis/Orcamento_PTL.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Módulo Q — display de QUANTIDADE (3 dígitos) + botão com LED, um por endereço de alto giro (andares 0 a 3).</t>
   </si>
   <si>
-    <t xml:space="preserve">Módulo E+Q — display de ENDEREÇO (8 dígitos) + QUANTIDADE (3 dígitos) + botão; usado nos andares 4 e 5 do alto giro (1 por andar em cada lado: 4 por estação) e em cada zona de baixo giro.</t>
+    <t xml:space="preserve">Módulo E+Q — display de ENDEREÇO (8 dígitos) + QUANTIDADE (3 dígitos) + botão; usado nos andares 4 e 5 do alto giro (1 por andar em cada lado: 4 por estação) e em cada zona de baixo giro (4 zonas por lado do corredor, na altura dos olhos).</t>
   </si>
   <si>
     <t xml:space="preserve">Nó de coluna — microcontrolador por coluna (prédio) do alto giro que liga os Módulos Q daquela coluna ao barramento RS-485.</t>
@@ -561,7 +561,7 @@
     <t xml:space="preserve">Coluna D (Piloto) = quantidade de estações nas linhas de total. Fonte: wms_endereco (cd_esteira 1 e 2), exportado em 23/10/2026; rua 90 (Marketing/Almoxarifado) desconsiderada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Regras: Alto giro = prédios 001-010; andares 4-5 com 4 displays E+Q por estação (A4 e A5 nos lados 001-005 e 006-010). Baixo giro = demais prédios (corredor, 015 e esquinas), 1 zona E+Q a cada 4 prédios.</t>
+    <t xml:space="preserve">Regras: Alto giro = prédios 001-010; andares 4-5 com 4 displays E+Q por estação (A4 e A5 nos lados 001-005 e 006-010). Baixo giro = demais prédios (corredor, 015 e esquinas): 4 zonas E+Q por lado do corredor; esquinas com zonas de 4 prédios.</t>
   </si>
   <si>
     <t xml:space="preserve">Código</t>
@@ -2404,15 +2404,15 @@
       </c>
       <c r="C4" s="10" t="n">
         <f aca="false">'A-Interno'!F13</f>
-        <v>10993.9714446721</v>
+        <v>11668.4916741803</v>
       </c>
       <c r="D4" s="10" t="n">
         <f aca="false">'A-Interno'!G13</f>
-        <v>199238.884893443</v>
+        <v>210828.961811475</v>
       </c>
       <c r="E4" s="11" t="n">
         <f aca="false">D4/Estações!$O$43</f>
-        <v>4980.97212233607</v>
+        <v>5270.72404528689</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2424,15 +2424,15 @@
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">'A-Interno'!F30</f>
-        <v>10873.0314446721</v>
+        <v>11507.5516741803</v>
       </c>
       <c r="D5" s="10" t="n">
         <f aca="false">'A-Interno'!G30</f>
-        <v>196955.764893443</v>
+        <v>207865.841811475</v>
       </c>
       <c r="E5" s="11" t="n">
         <f aca="false">D5/Estações!$O$43</f>
-        <v>4923.89412233607</v>
+        <v>5196.64604528689</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2444,15 +2444,15 @@
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">'A-Interno'!F24</f>
-        <v>14565.6204017273</v>
+        <v>15414.7933919717</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">'A-Interno'!G24</f>
-        <v>269763.669678719</v>
+        <v>284322.843529267</v>
       </c>
       <c r="E6" s="11" t="n">
         <f aca="false">D6/Estações!$O$43</f>
-        <v>6744.09174196797</v>
+        <v>7108.07108823167</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2464,15 +2464,15 @@
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">'A-Terceiros'!F10</f>
-        <v>32808.1033114633</v>
+        <v>34026.5052409715</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">'A-Terceiros'!G10</f>
-        <v>347860.285788283</v>
+        <v>368696.351606316</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">D7/Estações!$O$43</f>
-        <v>8696.50714470708</v>
+        <v>9217.4087901579</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2484,15 +2484,15 @@
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">'A-Terceiros'!F20</f>
-        <v>43195.6421514633</v>
+        <v>46363.4151309715</v>
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">'A-Terceiros'!G20</f>
-        <v>852329.779238283</v>
+        <v>906305.152906316</v>
       </c>
       <c r="E8" s="11" t="n">
         <f aca="false">D8/Estações!$O$43</f>
-        <v>21308.2444809571</v>
+        <v>22657.6288226579</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2504,15 +2504,15 @@
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">'B-RFID'!F10</f>
-        <v>15895.69987003</v>
+        <v>16744.8728602744</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">'B-RFID'!G10</f>
-        <v>294206.029106122</v>
+        <v>308765.20295667</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">D9/Estações!$O$43</f>
-        <v>7355.15072765304</v>
+        <v>7719.13007391674</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2524,15 +2524,15 @@
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">'B-RFID'!F15</f>
-        <v>15738.4231185465</v>
+        <v>16587.5961087909</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">'B-RFID'!G15</f>
-        <v>293219.724015103</v>
+        <v>307778.897865651</v>
       </c>
       <c r="E10" s="11" t="n">
         <f aca="false">D10/Estações!$O$43</f>
-        <v>7330.49310037757</v>
+        <v>7694.47244664127</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3045,7 +3045,7 @@
         <v>82</v>
       </c>
       <c r="J2" s="21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2" s="21" t="n">
         <v>10</v>
@@ -3055,11 +3055,11 @@
       </c>
       <c r="M2" s="22" t="n">
         <f aca="false">H2+J2</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N2" s="22" t="n">
         <f aca="false">K2+M2+2</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O2" s="21" t="n">
         <v>1</v>
@@ -3094,7 +3094,7 @@
         <v>156</v>
       </c>
       <c r="J3" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K3" s="21" t="n">
         <v>10</v>
@@ -3104,11 +3104,11 @@
       </c>
       <c r="M3" s="22" t="n">
         <f aca="false">H3+J3</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N3" s="22" t="n">
         <f aca="false">K3+M3+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O3" s="21" t="n">
         <v>1</v>
@@ -3143,7 +3143,7 @@
         <v>160</v>
       </c>
       <c r="J4" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K4" s="21" t="n">
         <v>10</v>
@@ -3153,11 +3153,11 @@
       </c>
       <c r="M4" s="22" t="n">
         <f aca="false">H4+J4</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N4" s="22" t="n">
         <f aca="false">K4+M4+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O4" s="21" t="n">
         <v>1</v>
@@ -3192,7 +3192,7 @@
         <v>160</v>
       </c>
       <c r="J5" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K5" s="21" t="n">
         <v>10</v>
@@ -3202,11 +3202,11 @@
       </c>
       <c r="M5" s="22" t="n">
         <f aca="false">H5+J5</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N5" s="22" t="n">
         <f aca="false">K5+M5+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>1</v>
@@ -3241,7 +3241,7 @@
         <v>160</v>
       </c>
       <c r="J6" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K6" s="21" t="n">
         <v>10</v>
@@ -3251,11 +3251,11 @@
       </c>
       <c r="M6" s="22" t="n">
         <f aca="false">H6+J6</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N6" s="22" t="n">
         <f aca="false">K6+M6+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>1</v>
@@ -3290,7 +3290,7 @@
         <v>160</v>
       </c>
       <c r="J7" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K7" s="21" t="n">
         <v>10</v>
@@ -3300,11 +3300,11 @@
       </c>
       <c r="M7" s="22" t="n">
         <f aca="false">H7+J7</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N7" s="22" t="n">
         <f aca="false">K7+M7+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>1</v>
@@ -3339,7 +3339,7 @@
         <v>192</v>
       </c>
       <c r="J8" s="21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K8" s="21" t="n">
         <v>10</v>
@@ -3349,11 +3349,11 @@
       </c>
       <c r="M8" s="22" t="n">
         <f aca="false">H8+J8</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N8" s="22" t="n">
         <f aca="false">K8+M8+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>1</v>
@@ -3388,7 +3388,7 @@
         <v>188</v>
       </c>
       <c r="J9" s="21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K9" s="21" t="n">
         <v>10</v>
@@ -3398,11 +3398,11 @@
       </c>
       <c r="M9" s="22" t="n">
         <f aca="false">H9+J9</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N9" s="22" t="n">
         <f aca="false">K9+M9+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>1</v>
@@ -3437,7 +3437,7 @@
         <v>160</v>
       </c>
       <c r="J10" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K10" s="21" t="n">
         <v>10</v>
@@ -3447,11 +3447,11 @@
       </c>
       <c r="M10" s="22" t="n">
         <f aca="false">H10+J10</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N10" s="22" t="n">
         <f aca="false">K10+M10+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>1</v>
@@ -3486,7 +3486,7 @@
         <v>160</v>
       </c>
       <c r="J11" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K11" s="21" t="n">
         <v>10</v>
@@ -3496,11 +3496,11 @@
       </c>
       <c r="M11" s="22" t="n">
         <f aca="false">H11+J11</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N11" s="22" t="n">
         <f aca="false">K11+M11+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>1</v>
@@ -3535,7 +3535,7 @@
         <v>160</v>
       </c>
       <c r="J12" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K12" s="21" t="n">
         <v>10</v>
@@ -3545,11 +3545,11 @@
       </c>
       <c r="M12" s="22" t="n">
         <f aca="false">H12+J12</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N12" s="22" t="n">
         <f aca="false">K12+M12+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1</v>
@@ -3584,7 +3584,7 @@
         <v>160</v>
       </c>
       <c r="J13" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K13" s="21" t="n">
         <v>10</v>
@@ -3594,11 +3594,11 @@
       </c>
       <c r="M13" s="22" t="n">
         <f aca="false">H13+J13</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N13" s="22" t="n">
         <f aca="false">K13+M13+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1</v>
@@ -3633,7 +3633,7 @@
         <v>192</v>
       </c>
       <c r="J14" s="21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K14" s="21" t="n">
         <v>10</v>
@@ -3643,11 +3643,11 @@
       </c>
       <c r="M14" s="22" t="n">
         <f aca="false">H14+J14</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N14" s="22" t="n">
         <f aca="false">K14+M14+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>1</v>
@@ -3682,7 +3682,7 @@
         <v>188</v>
       </c>
       <c r="J15" s="21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K15" s="21" t="n">
         <v>10</v>
@@ -3692,11 +3692,11 @@
       </c>
       <c r="M15" s="22" t="n">
         <f aca="false">H15+J15</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N15" s="22" t="n">
         <f aca="false">K15+M15+2</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O15" s="21" t="n">
         <v>1</v>
@@ -3731,7 +3731,7 @@
         <v>160</v>
       </c>
       <c r="J16" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K16" s="21" t="n">
         <v>10</v>
@@ -3741,11 +3741,11 @@
       </c>
       <c r="M16" s="22" t="n">
         <f aca="false">H16+J16</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N16" s="22" t="n">
         <f aca="false">K16+M16+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O16" s="21" t="n">
         <v>1</v>
@@ -3780,7 +3780,7 @@
         <v>160</v>
       </c>
       <c r="J17" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K17" s="21" t="n">
         <v>10</v>
@@ -3790,11 +3790,11 @@
       </c>
       <c r="M17" s="22" t="n">
         <f aca="false">H17+J17</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N17" s="22" t="n">
         <f aca="false">K17+M17+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O17" s="21" t="n">
         <v>1</v>
@@ -3829,7 +3829,7 @@
         <v>160</v>
       </c>
       <c r="J18" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K18" s="21" t="n">
         <v>10</v>
@@ -3839,11 +3839,11 @@
       </c>
       <c r="M18" s="22" t="n">
         <f aca="false">H18+J18</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N18" s="22" t="n">
         <f aca="false">K18+M18+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O18" s="21" t="n">
         <v>1</v>
@@ -3878,7 +3878,7 @@
         <v>160</v>
       </c>
       <c r="J19" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K19" s="21" t="n">
         <v>10</v>
@@ -3888,11 +3888,11 @@
       </c>
       <c r="M19" s="22" t="n">
         <f aca="false">H19+J19</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N19" s="22" t="n">
         <f aca="false">K19+M19+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O19" s="21" t="n">
         <v>1</v>
@@ -3927,7 +3927,7 @@
         <v>160</v>
       </c>
       <c r="J20" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K20" s="21" t="n">
         <v>10</v>
@@ -3937,11 +3937,11 @@
       </c>
       <c r="M20" s="22" t="n">
         <f aca="false">H20+J20</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N20" s="22" t="n">
         <f aca="false">K20+M20+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O20" s="21" t="n">
         <v>1</v>
@@ -4025,7 +4025,7 @@
         <v>128</v>
       </c>
       <c r="J22" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K22" s="21" t="n">
         <v>10</v>
@@ -4035,11 +4035,11 @@
       </c>
       <c r="M22" s="22" t="n">
         <f aca="false">H22+J22</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N22" s="22" t="n">
         <f aca="false">K22+M22+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O22" s="21" t="n">
         <v>1</v>
@@ -4074,7 +4074,7 @@
         <v>131</v>
       </c>
       <c r="J23" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K23" s="21" t="n">
         <v>10</v>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="M23" s="22" t="n">
         <f aca="false">H23+J23</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N23" s="22" t="n">
         <f aca="false">K23+M23+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O23" s="21" t="n">
         <v>1</v>
@@ -4123,7 +4123,7 @@
         <v>131</v>
       </c>
       <c r="J24" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K24" s="21" t="n">
         <v>10</v>
@@ -4133,11 +4133,11 @@
       </c>
       <c r="M24" s="22" t="n">
         <f aca="false">H24+J24</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N24" s="22" t="n">
         <f aca="false">K24+M24+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O24" s="21" t="n">
         <v>1</v>
@@ -4172,7 +4172,7 @@
         <v>131</v>
       </c>
       <c r="J25" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K25" s="21" t="n">
         <v>10</v>
@@ -4182,11 +4182,11 @@
       </c>
       <c r="M25" s="22" t="n">
         <f aca="false">H25+J25</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N25" s="22" t="n">
         <f aca="false">K25+M25+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O25" s="21" t="n">
         <v>1</v>
@@ -4221,7 +4221,7 @@
         <v>131</v>
       </c>
       <c r="J26" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K26" s="21" t="n">
         <v>10</v>
@@ -4231,11 +4231,11 @@
       </c>
       <c r="M26" s="22" t="n">
         <f aca="false">H26+J26</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N26" s="22" t="n">
         <f aca="false">K26+M26+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O26" s="21" t="n">
         <v>1</v>
@@ -4270,7 +4270,7 @@
         <v>131</v>
       </c>
       <c r="J27" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K27" s="21" t="n">
         <v>10</v>
@@ -4280,11 +4280,11 @@
       </c>
       <c r="M27" s="22" t="n">
         <f aca="false">H27+J27</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N27" s="22" t="n">
         <f aca="false">K27+M27+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O27" s="21" t="n">
         <v>1</v>
@@ -4319,7 +4319,7 @@
         <v>230</v>
       </c>
       <c r="J28" s="21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K28" s="21" t="n">
         <v>10</v>
@@ -4329,11 +4329,11 @@
       </c>
       <c r="M28" s="22" t="n">
         <f aca="false">H28+J28</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N28" s="22" t="n">
         <f aca="false">K28+M28+2</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O28" s="21" t="n">
         <v>1</v>
@@ -4368,7 +4368,7 @@
         <v>227</v>
       </c>
       <c r="J29" s="21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K29" s="21" t="n">
         <v>10</v>
@@ -4378,11 +4378,11 @@
       </c>
       <c r="M29" s="22" t="n">
         <f aca="false">H29+J29</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N29" s="22" t="n">
         <f aca="false">K29+M29+2</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O29" s="21" t="n">
         <v>1</v>
@@ -4417,7 +4417,7 @@
         <v>131</v>
       </c>
       <c r="J30" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K30" s="21" t="n">
         <v>10</v>
@@ -4427,11 +4427,11 @@
       </c>
       <c r="M30" s="22" t="n">
         <f aca="false">H30+J30</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N30" s="22" t="n">
         <f aca="false">K30+M30+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O30" s="21" t="n">
         <v>1</v>
@@ -4466,7 +4466,7 @@
         <v>131</v>
       </c>
       <c r="J31" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K31" s="21" t="n">
         <v>10</v>
@@ -4476,11 +4476,11 @@
       </c>
       <c r="M31" s="22" t="n">
         <f aca="false">H31+J31</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N31" s="22" t="n">
         <f aca="false">K31+M31+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O31" s="21" t="n">
         <v>1</v>
@@ -4515,7 +4515,7 @@
         <v>131</v>
       </c>
       <c r="J32" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K32" s="21" t="n">
         <v>10</v>
@@ -4525,11 +4525,11 @@
       </c>
       <c r="M32" s="22" t="n">
         <f aca="false">H32+J32</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N32" s="22" t="n">
         <f aca="false">K32+M32+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O32" s="21" t="n">
         <v>1</v>
@@ -4564,7 +4564,7 @@
         <v>131</v>
       </c>
       <c r="J33" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K33" s="21" t="n">
         <v>10</v>
@@ -4574,11 +4574,11 @@
       </c>
       <c r="M33" s="22" t="n">
         <f aca="false">H33+J33</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N33" s="22" t="n">
         <f aca="false">K33+M33+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O33" s="21" t="n">
         <v>1</v>
@@ -4613,7 +4613,7 @@
         <v>230</v>
       </c>
       <c r="J34" s="21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K34" s="21" t="n">
         <v>10</v>
@@ -4623,11 +4623,11 @@
       </c>
       <c r="M34" s="22" t="n">
         <f aca="false">H34+J34</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N34" s="22" t="n">
         <f aca="false">K34+M34+2</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O34" s="21" t="n">
         <v>1</v>
@@ -4662,7 +4662,7 @@
         <v>227</v>
       </c>
       <c r="J35" s="21" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K35" s="21" t="n">
         <v>10</v>
@@ -4672,11 +4672,11 @@
       </c>
       <c r="M35" s="22" t="n">
         <f aca="false">H35+J35</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N35" s="22" t="n">
         <f aca="false">K35+M35+2</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O35" s="21" t="n">
         <v>1</v>
@@ -4711,7 +4711,7 @@
         <v>131</v>
       </c>
       <c r="J36" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K36" s="21" t="n">
         <v>10</v>
@@ -4721,11 +4721,11 @@
       </c>
       <c r="M36" s="22" t="n">
         <f aca="false">H36+J36</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N36" s="22" t="n">
         <f aca="false">K36+M36+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O36" s="21" t="n">
         <v>1</v>
@@ -4760,7 +4760,7 @@
         <v>131</v>
       </c>
       <c r="J37" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K37" s="21" t="n">
         <v>10</v>
@@ -4770,11 +4770,11 @@
       </c>
       <c r="M37" s="22" t="n">
         <f aca="false">H37+J37</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N37" s="22" t="n">
         <f aca="false">K37+M37+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O37" s="21" t="n">
         <v>1</v>
@@ -4809,7 +4809,7 @@
         <v>131</v>
       </c>
       <c r="J38" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K38" s="21" t="n">
         <v>10</v>
@@ -4819,11 +4819,11 @@
       </c>
       <c r="M38" s="22" t="n">
         <f aca="false">H38+J38</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N38" s="22" t="n">
         <f aca="false">K38+M38+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O38" s="21" t="n">
         <v>1</v>
@@ -4858,7 +4858,7 @@
         <v>131</v>
       </c>
       <c r="J39" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K39" s="21" t="n">
         <v>10</v>
@@ -4868,11 +4868,11 @@
       </c>
       <c r="M39" s="22" t="n">
         <f aca="false">H39+J39</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N39" s="22" t="n">
         <f aca="false">K39+M39+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O39" s="21" t="n">
         <v>1</v>
@@ -4907,7 +4907,7 @@
         <v>131</v>
       </c>
       <c r="J40" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K40" s="21" t="n">
         <v>10</v>
@@ -4917,11 +4917,11 @@
       </c>
       <c r="M40" s="22" t="n">
         <f aca="false">H40+J40</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N40" s="22" t="n">
         <f aca="false">K40+M40+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O40" s="21" t="n">
         <v>1</v>
@@ -4956,7 +4956,7 @@
         <v>131</v>
       </c>
       <c r="J41" s="21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K41" s="21" t="n">
         <v>10</v>
@@ -4966,11 +4966,11 @@
       </c>
       <c r="M41" s="22" t="n">
         <f aca="false">H41+J41</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N41" s="22" t="n">
         <f aca="false">K41+M41+2</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O41" s="21" t="n">
         <v>1</v>
@@ -5006,7 +5006,7 @@
       </c>
       <c r="J43" s="25" t="n">
         <f aca="false">SUM(J2:J41)</f>
-        <v>248</v>
+        <v>325</v>
       </c>
       <c r="K43" s="25" t="n">
         <f aca="false">SUM(K2:K41)</f>
@@ -5018,11 +5018,11 @@
       </c>
       <c r="M43" s="25" t="n">
         <f aca="false">SUM(M2:M41)</f>
-        <v>408</v>
+        <v>485</v>
       </c>
       <c r="N43" s="25" t="n">
         <f aca="false">SUM(N2:N41)</f>
-        <v>888</v>
+        <v>965</v>
       </c>
       <c r="O43" s="25" t="n">
         <f aca="false">SUM(O2:O41)</f>
@@ -5059,7 +5059,7 @@
       </c>
       <c r="J44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",J2:J41)</f>
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",K2:K41)</f>
@@ -5071,11 +5071,11 @@
       </c>
       <c r="M44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",M2:M41)</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",N2:N41)</f>
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="O44" s="25" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",O2:O41)</f>
@@ -7285,11 +7285,11 @@
       </c>
       <c r="C5" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$14),0)</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D5" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$43*(1+Premissas!$B$14),0)</f>
-        <v>449</v>
+        <v>534</v>
       </c>
       <c r="E5" s="33" t="n">
         <f aca="false">Composição!$F$27</f>
@@ -7297,11 +7297,11 @@
       </c>
       <c r="F5" s="27" t="n">
         <f aca="false">C5*E5</f>
-        <v>2726.9</v>
+        <v>3346.65</v>
       </c>
       <c r="G5" s="27" t="n">
         <f aca="false">D5*E5</f>
-        <v>55653.55</v>
+        <v>66189.3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7341,11 +7341,11 @@
       </c>
       <c r="C7" s="37" t="n">
         <f aca="false">Estações!$N$44*Premissas!$B$15</f>
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="D7" s="37" t="n">
         <f aca="false">Estações!$N$43*Premissas!$B$15</f>
-        <v>2664</v>
+        <v>2895</v>
       </c>
       <c r="E7" s="33" t="n">
         <f aca="false">Preços!$D$13</f>
@@ -7353,11 +7353,11 @@
       </c>
       <c r="F7" s="27" t="n">
         <f aca="false">C7*E7</f>
-        <v>532.072524590164</v>
+        <v>580.442754098361</v>
       </c>
       <c r="G7" s="27" t="n">
         <f aca="false">D7*E7</f>
-        <v>10738.1909508197</v>
+        <v>11669.3178688525</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7369,11 +7369,11 @@
       </c>
       <c r="C8" s="37" t="n">
         <f aca="false">Estações!$N$44*2</f>
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D8" s="37" t="n">
         <f aca="false">Estações!$N$43*2</f>
-        <v>1776</v>
+        <v>1930</v>
       </c>
       <c r="E8" s="33" t="n">
         <f aca="false">Preços!$D$12</f>
@@ -7381,11 +7381,11 @@
       </c>
       <c r="F8" s="27" t="n">
         <f aca="false">C8*E8</f>
-        <v>70.4</v>
+        <v>76.8</v>
       </c>
       <c r="G8" s="27" t="n">
         <f aca="false">D8*E8</f>
-        <v>1420.8</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7510,11 +7510,11 @@
       <c r="E13" s="35"/>
       <c r="F13" s="36" t="n">
         <f aca="false">SUM(F3:F12)</f>
-        <v>10993.9714446721</v>
+        <v>11668.4916741803</v>
       </c>
       <c r="G13" s="36" t="n">
         <f aca="false">SUM(G3:G12)</f>
-        <v>199238.884893443</v>
+        <v>210828.961811475</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7587,11 +7587,11 @@
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">C5*Premissas!$B$10</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">D5*Premissas!$B$10</f>
-        <v>449</v>
+        <v>534</v>
       </c>
       <c r="E18" s="33" t="n">
         <f aca="false">Premissas!$B$7</f>
@@ -7599,11 +7599,11 @@
       </c>
       <c r="F18" s="27" t="n">
         <f aca="false">C18*E18</f>
-        <v>768.472147239264</v>
+        <v>943.12490797546</v>
       </c>
       <c r="G18" s="27" t="n">
         <f aca="false">D18*E18</f>
-        <v>15683.8179141104</v>
+        <v>18652.9148466258</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7697,20 +7697,20 @@
       <c r="B22" s="35"/>
       <c r="C22" s="38" t="n">
         <f aca="false">SUM(C16:C21)</f>
-        <v>102.25</v>
+        <v>107.25</v>
       </c>
       <c r="D22" s="38" t="n">
         <f aca="false">SUM(D16:D21)</f>
-        <v>2019</v>
+        <v>2104</v>
       </c>
       <c r="E22" s="35"/>
       <c r="F22" s="36" t="n">
         <f aca="false">SUM(F16:F21)</f>
-        <v>3571.64895705522</v>
+        <v>3746.30171779141</v>
       </c>
       <c r="G22" s="36" t="n">
         <f aca="false">SUM(G16:G21)</f>
-        <v>70524.7847852761</v>
+        <v>73493.8817177914</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7723,11 +7723,11 @@
       <c r="E24" s="35"/>
       <c r="F24" s="36" t="n">
         <f aca="false">F13+F22</f>
-        <v>14565.6204017273</v>
+        <v>15414.7933919717</v>
       </c>
       <c r="G24" s="36" t="n">
         <f aca="false">G13+G22</f>
-        <v>269763.669678719</v>
+        <v>284322.843529267</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7744,11 +7744,11 @@
       </c>
       <c r="C27" s="37" t="n">
         <f aca="false">-(C4+C5+C6)</f>
-        <v>-47</v>
+        <v>-52</v>
       </c>
       <c r="D27" s="37" t="n">
         <f aca="false">-(D4+D5+D6)</f>
-        <v>-933</v>
+        <v>-1018</v>
       </c>
       <c r="E27" s="33" t="n">
         <f aca="false">Preços!$D$9</f>
@@ -7756,11 +7756,11 @@
       </c>
       <c r="F27" s="27" t="n">
         <f aca="false">C27*E27</f>
-        <v>-376</v>
+        <v>-416</v>
       </c>
       <c r="G27" s="27" t="n">
         <f aca="false">D27*E27</f>
-        <v>-7464</v>
+        <v>-8144</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7829,11 +7829,11 @@
       <c r="E30" s="35"/>
       <c r="F30" s="36" t="n">
         <f aca="false">F13+SUM(F27:F29)</f>
-        <v>10873.0314446721</v>
+        <v>11507.5516741803</v>
       </c>
       <c r="G30" s="36" t="n">
         <f aca="false">G13+SUM(G27:G29)</f>
-        <v>196955.764893443</v>
+        <v>207865.841811475</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7961,11 +7961,11 @@
       </c>
       <c r="C4" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$14),0)</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D4" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$43*(1+Premissas!$B$14),0)</f>
-        <v>449</v>
+        <v>534</v>
       </c>
       <c r="E4" s="33" t="n">
         <f aca="false">Preços!$D$34+Preços!$D$15+Preços!$D$10</f>
@@ -7973,11 +7973,11 @@
       </c>
       <c r="F4" s="27" t="n">
         <f aca="false">C4*E4</f>
-        <v>5119.97948</v>
+        <v>6283.61118</v>
       </c>
       <c r="G4" s="27" t="n">
         <f aca="false">D4*E4</f>
-        <v>104494.12666</v>
+        <v>124275.86556</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8017,11 +8017,11 @@
       </c>
       <c r="C6" s="37" t="n">
         <f aca="false">(Estações!$F$44+Estações!$M$44)*Premissas!$B$15</f>
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D6" s="37" t="n">
         <f aca="false">(Estações!$F$43+Estações!$M$43)*Premissas!$B$15</f>
-        <v>5064</v>
+        <v>5295</v>
       </c>
       <c r="E6" s="33" t="n">
         <f aca="false">Preços!$D$13+2*Preços!$D$12/Premissas!$B$15</f>
@@ -8029,11 +8029,11 @@
       </c>
       <c r="F6" s="27" t="n">
         <f aca="false">C6*E6</f>
-        <v>1150.17481967213</v>
+        <v>1204.94504918033</v>
       </c>
       <c r="G6" s="27" t="n">
         <f aca="false">D6*E6</f>
-        <v>23113.036852459</v>
+        <v>24167.3637704918</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8123,11 +8123,11 @@
       <c r="E10" s="35"/>
       <c r="F10" s="36" t="n">
         <f aca="false">SUM(F3:F9)</f>
-        <v>32808.1033114633</v>
+        <v>34026.5052409715</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">SUM(G3:G9)</f>
-        <v>347860.285788283</v>
+        <v>368696.351606316</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8172,11 +8172,11 @@
       </c>
       <c r="C14" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$14),0)</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D14" s="37" t="n">
         <f aca="false">ROUNDUP(Estações!$M$43*(1+Premissas!$B$14),0)</f>
-        <v>449</v>
+        <v>534</v>
       </c>
       <c r="E14" s="33" t="n">
         <f aca="false">Preços!$D$31</f>
@@ -8184,11 +8184,11 @@
       </c>
       <c r="F14" s="27" t="n">
         <f aca="false">C14*E14</f>
-        <v>13697.2121</v>
+        <v>16810.21485</v>
       </c>
       <c r="G14" s="27" t="n">
         <f aca="false">D14*E14</f>
-        <v>279547.64695</v>
+        <v>332468.6937</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8256,11 +8256,11 @@
       </c>
       <c r="C17" s="37" t="n">
         <f aca="false">(Estações!$F$44+Estações!$M$44)*Premissas!$B$15</f>
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D17" s="37" t="n">
         <f aca="false">(Estações!$F$43+Estações!$M$43)*Premissas!$B$15</f>
-        <v>5064</v>
+        <v>5295</v>
       </c>
       <c r="E17" s="33" t="n">
         <f aca="false">Preços!$D$13+2*Preços!$D$12/Premissas!$B$15</f>
@@ -8268,11 +8268,11 @@
       </c>
       <c r="F17" s="27" t="n">
         <f aca="false">C17*E17</f>
-        <v>1150.17481967213</v>
+        <v>1204.94504918033</v>
       </c>
       <c r="G17" s="27" t="n">
         <f aca="false">D17*E17</f>
-        <v>23113.036852459</v>
+        <v>24167.3637704918</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8336,11 +8336,11 @@
       <c r="E20" s="35"/>
       <c r="F20" s="36" t="n">
         <f aca="false">SUM(F13:F19)</f>
-        <v>43195.6421514633</v>
+        <v>46363.4151309715</v>
       </c>
       <c r="G20" s="36" t="n">
         <f aca="false">SUM(G13:G19)</f>
-        <v>852329.779238283</v>
+        <v>906305.152906316</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8416,11 +8416,11 @@
       <c r="E3" s="13"/>
       <c r="F3" s="33" t="n">
         <f aca="false">'A-Interno'!F24</f>
-        <v>14565.6204017273</v>
+        <v>15414.7933919717</v>
       </c>
       <c r="G3" s="33" t="n">
         <f aca="false">'A-Interno'!G24</f>
-        <v>269763.669678719</v>
+        <v>284322.843529267</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8550,11 +8550,11 @@
       <c r="E10" s="35"/>
       <c r="F10" s="36" t="n">
         <f aca="false">F3+F4+F5+F8+F9</f>
-        <v>15895.69987003</v>
+        <v>16744.8728602744</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">G3+G4+G5+G8+G9</f>
-        <v>294206.029106122</v>
+        <v>308765.20295667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8628,11 +8628,11 @@
       <c r="E15" s="35"/>
       <c r="F15" s="36" t="n">
         <f aca="false">F3+F4+F5+F13+F14</f>
-        <v>15738.4231185465</v>
+        <v>16587.5961087909</v>
       </c>
       <c r="G15" s="36" t="n">
         <f aca="false">G3+G4+G5+G13+G14</f>
-        <v>293219.724015103</v>
+        <v>307778.897865651</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Textos revisados e diagrama de componentes
- documento técnico, apresentação e planilha com linguagem mais direta
- novo diagrama de arquitetura de componentes (documento e apresentação)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TBWA3G7ku1j3oTf4VMkLud
</commit_message>
<xml_diff>
--- a/projeto/entregaveis/Orcamento_PTL.xlsx
+++ b/projeto/entregaveis/Orcamento_PTL.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="433">
   <si>
-    <t xml:space="preserve">Orçamento — Projeto Pick-to-Light (Flow Rack)</t>
+    <t xml:space="preserve">Orçamento do projeto Pick-to-Light (flow rack)</t>
   </si>
   <si>
     <t xml:space="preserve">Arquitetura A (coletor + concentrador + displays) e Arquitetura B (identificação por RFID)</t>
@@ -40,13 +40,13 @@
     <t xml:space="preserve">COMO USAR</t>
   </si>
   <si>
-    <t xml:space="preserve">• Células em AZUL são entradas editáveis (quantidades, preços, premissas). Células em PRETO são fórmulas — não editar.</t>
+    <t xml:space="preserve">• Células em AZUL são entradas editáveis (quantidades, preços, premissas). Células em PRETO são fórmulas: não editar.</t>
   </si>
   <si>
     <t xml:space="preserve">• Células com fundo AMARELO são premissas/estimativas que precisam de cotação ou confirmação.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Aba 'Estações': números de endereços por estação, extraídos de wms_endereco (esteiras 1 e 2) em 23/10/2026. Corrija qualquer número direto ali — todo o orçamento recalcula.</t>
+    <t xml:space="preserve">• Aba 'Estações': números de endereços por estação, extraídos de wms_endereco (esteiras 1 e 2) em 23/10/2026. Corrija qualquer número direto ali: todo o orçamento recalcula.</t>
   </si>
   <si>
     <t xml:space="preserve">• Coluna 'Piloto' (S/N) na aba 'Estações' define quais estações entram no cenário piloto (padrão: 05 e 27).</t>
@@ -58,52 +58,52 @@
     <t xml:space="preserve">ABAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Premissas — câmbio, fator de importação, custo-hora, horas de montagem/instalação, reserva técnica, frota de caixas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estações — dimensionamento por estação (40 estações: 20 Medicamento + 20 Perfumaria).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preços — catálogo de peças com fonte.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Composição — lista de materiais (BOM) de cada tipo de módulo e custo unitário.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A-Interno — Arquitetura A com produção interna: peças, peças + mão de obra, variante 5 V.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A-Terceiros — Arquitetura A com produção de terceiros: (T1) placa própria montada por EMS e (T2) PTL comercial importado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B-RFID — Arquitetura B: mesma infraestrutura de displays + identificação RFID (B1 pulseira, B2 leitor fixo).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Software — esforço estimado de desenvolvimento (horas) para as duas arquiteturas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumo — comparativo de todos os cenários: Piloto x Operação completa.</t>
+    <t xml:space="preserve">Premissas: câmbio, fator de importação, custo-hora, horas de montagem/instalação, reserva técnica, frota de caixas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estações: dimensionamento por estação (40 estações: 20 Medicamento + 20 Perfumaria).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preços: catálogo de peças com fonte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Composição: lista de materiais (BOM) de cada tipo de módulo e custo unitário.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-Interno: Arquitetura A com produção interna: peças, peças + mão de obra, variante 5 V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-Terceiros: Arquitetura A com produção de terceiros: (T1) placa própria montada por EMS e (T2) PTL comercial importado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-RFID: Arquitetura B: mesma infraestrutura de displays + identificação RFID (B1 pulseira, B2 leitor fixo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software: esforço estimado de desenvolvimento (horas) para as duas arquiteturas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumo: comparativo de todos os cenários: Piloto x Operação completa.</t>
   </si>
   <si>
     <t xml:space="preserve">TERMOS</t>
   </si>
   <si>
-    <t xml:space="preserve">Módulo Q — display de QUANTIDADE (3 dígitos) + botão com LED, um por endereço de alto giro (andares 0 a 3).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Módulo E+Q — display de ENDEREÇO (8 dígitos) + QUANTIDADE (3 dígitos) + botão; usado nos andares 4 e 5 do alto giro (1 por andar em cada lado: 4 por estação) e em cada zona de baixo giro (4 zonas por lado do corredor, na altura dos olhos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nó de coluna — microcontrolador por coluna (prédio) do alto giro que liga os Módulos Q daquela coluna ao barramento RS-485.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concentrador — controlador da estação (Ethernet cabeada), recebe a caixa do serviço PTL e comanda os barramentos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zona de baixo giro — 1 display E+Q a cada 4 prédios do fundo (inclui prédio 015 na 1ª zona e prédios de esquina).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumo do orçamento — Pick-to-Light</t>
+    <t xml:space="preserve">Módulo Q: display de QUANTIDADE (3 dígitos) + botão com LED, um por endereço de alto giro (andares 0 a 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulo E+Q: display de ENDEREÇO (8 dígitos) + QUANTIDADE (3 dígitos) + botão; usado nos andares 4 e 5 do alto giro (1 por andar em cada lado: 4 por estação) e em cada zona de baixo giro (4 zonas por lado do corredor, na altura dos olhos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nó de coluna: microcontrolador por coluna (prédio) do alto giro que liga os Módulos Q daquela coluna ao barramento RS-485.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentrador: controlador da estação (Ethernet cabeada), recebe a caixa do serviço PTL e comanda os barramentos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zona de baixo giro: 4 zonas por lado do corredor, cada uma com 1 display E+Q na altura dos olhos (o prédio 015 entra na zona D1; esquinas têm zonas de 4 prédios).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumo do orçamento, Pick-to-Light</t>
   </si>
   <si>
     <t xml:space="preserve">Piloto: estações marcadas 'S' na aba Estações (padrão 05 e 27). Valores de hardware; software na última linha.</t>
@@ -121,52 +121,52 @@
     <t xml:space="preserve">Operação completa (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Por estação — completo (R$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A — Interno, só peças (12 V)</t>
+    <t xml:space="preserve">Por estação, completo (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A interno, só peças (12 V)</t>
   </si>
   <si>
     <t xml:space="preserve">Peças para toda a operação, montagem própria</t>
   </si>
   <si>
-    <t xml:space="preserve">A — Interno, só peças (variante 5 V)</t>
+    <t xml:space="preserve">A interno, só peças (variante 5 V)</t>
   </si>
   <si>
     <t xml:space="preserve">Sem reguladores, fonte 5 V, mais cabo de força</t>
   </si>
   <si>
-    <t xml:space="preserve">A — Interno, peças + mão de obra</t>
+    <t xml:space="preserve">A interno, peças + mão de obra</t>
   </si>
   <si>
     <t xml:space="preserve">Montagem, instalação e comissionamento internos</t>
   </si>
   <si>
-    <t xml:space="preserve">A — Terceiros T1 (PCB própria via EMS)</t>
+    <t xml:space="preserve">A terceiros, T1 (PCB própria via EMS)</t>
   </si>
   <si>
     <t xml:space="preserve">Placas próprias fabricadas/montadas por terceiros + instalação</t>
   </si>
   <si>
-    <t xml:space="preserve">A — Terceiros T2 (PTL comercial importado)</t>
+    <t xml:space="preserve">A terceiros, T2 (PTL comercial importado)</t>
   </si>
   <si>
     <t xml:space="preserve">Hardware PTL pronto + instalação</t>
   </si>
   <si>
-    <t xml:space="preserve">B1 — RFID com pulseira</t>
+    <t xml:space="preserve">B1, RFID com pulseira</t>
   </si>
   <si>
     <t xml:space="preserve">Displays (A interno) + tags + pulseiras NFC</t>
   </si>
   <si>
-    <t xml:space="preserve">B2 — RFID com leitor fixo na estação</t>
+    <t xml:space="preserve">B2, RFID com leitor fixo na estação</t>
   </si>
   <si>
     <t xml:space="preserve">Displays (A interno) + tags + leitor fixo e painel</t>
   </si>
   <si>
-    <t xml:space="preserve">Opcional — guia de coluna no baixo giro</t>
+    <t xml:space="preserve">Opcional, guia de coluna no baixo giro</t>
   </si>
   <si>
     <t xml:space="preserve">1 LED por prédio do fundo</t>
@@ -202,7 +202,7 @@
     <t xml:space="preserve">R$/US$</t>
   </si>
   <si>
-    <t xml:space="preserve">renovainvest.com.br/dolar-hoje — 23/10/2026 12h11</t>
+    <t xml:space="preserve">renovainvest.com.br/dolar-hoje, 23/10/2026 12h11</t>
   </si>
   <si>
     <t xml:space="preserve">Fator de importação (frete + impostos + despacho) sobre o valor FOB</t>
@@ -247,7 +247,7 @@
     <t xml:space="preserve">Fórmula: salário × encargos ÷ horas</t>
   </si>
   <si>
-    <t xml:space="preserve">Montagem — Módulo Q</t>
+    <t xml:space="preserve">Montagem, Módulo Q</t>
   </si>
   <si>
     <t xml:space="preserve">h/un</t>
@@ -256,19 +256,19 @@
     <t xml:space="preserve">Estimativa: display + botão + carcaça + teste</t>
   </si>
   <si>
-    <t xml:space="preserve">Montagem — Nó de coluna</t>
+    <t xml:space="preserve">Montagem, Nó de coluna</t>
   </si>
   <si>
     <t xml:space="preserve">Estimativa: placa base, soldas, gravação de firmware, teste</t>
   </si>
   <si>
-    <t xml:space="preserve">Montagem — Módulo E+Q</t>
+    <t xml:space="preserve">Montagem, Módulo E+Q</t>
   </si>
   <si>
     <t xml:space="preserve">Estimativa</t>
   </si>
   <si>
-    <t xml:space="preserve">Montagem — Concentrador (gabinete completo)</t>
+    <t xml:space="preserve">Montagem, Concentrador (gabinete completo)</t>
   </si>
   <si>
     <t xml:space="preserve">Instalação por estação (canaletas, módulos, cabos)</t>
@@ -358,7 +358,7 @@
     <t xml:space="preserve">R$/m</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa — cotar</t>
+    <t xml:space="preserve">Estimativa, cotar</t>
   </si>
   <si>
     <t xml:space="preserve">Rua (estação)</t>
@@ -552,10 +552,10 @@
     <t xml:space="preserve">45</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL — operação completa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL — piloto (Piloto = S)</t>
+    <t xml:space="preserve">Total da operação completa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total do piloto (Piloto = S)</t>
   </si>
   <si>
     <t xml:space="preserve">Coluna D (Piloto) = quantidade de estações nas linhas de total. Fonte: wms_endereco (cd_esteira 1 e 2), exportado em 23/10/2026; rua 90 (Marketing/Almoxarifado) desconsiderada.</t>
@@ -585,10 +585,10 @@
     <t xml:space="preserve">P01</t>
   </si>
   <si>
-    <t xml:space="preserve">Display 7 segmentos 4 dígitos TM1637 (usa 3 dígitos — quantidade)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usinainfo — Módulo Display TM1637 4 dígitos vermelho — 23/10/2026 (Pix)</t>
+    <t xml:space="preserve">Display 7 segmentos 4 dígitos TM1637 (usa 3 dígitos, quantidade)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usinainfo, Módulo Display TM1637 4 dígitos vermelho, 23/10/2026 (Pix)</t>
   </si>
   <si>
     <t xml:space="preserve">Cotado</t>
@@ -600,7 +600,7 @@
     <t xml:space="preserve">Display 7 segmentos 8 dígitos MAX7219 (endereço)</t>
   </si>
   <si>
-    <t xml:space="preserve">Usinainfo — Display MAX7219 8 dígitos SPI — 23/10/2026 (Pix)</t>
+    <t xml:space="preserve">Usinainfo, Display MAX7219 8 dígitos SPI, 23/10/2026 (Pix)</t>
   </si>
   <si>
     <t xml:space="preserve">P03</t>
@@ -609,7 +609,7 @@
     <t xml:space="preserve">Microcontrolador Raspberry Pi Pico (RP2040)</t>
   </si>
   <si>
-    <t xml:space="preserve">MakerHero — Raspberry Pi Pico — 23/10/2026</t>
+    <t xml:space="preserve">MakerHero, Raspberry Pi Pico, 23/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">P04</t>
@@ -618,7 +618,7 @@
     <t xml:space="preserve">Módulo transceptor RS-485 (MAX485)</t>
   </si>
   <si>
-    <t xml:space="preserve">Saravati — Módulo conversor TTL/RS485 MAX485 — 23/10/2026</t>
+    <t xml:space="preserve">Saravati, Módulo conversor TTL/RS485 MAX485, 23/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">P05</t>
@@ -627,7 +627,7 @@
     <t xml:space="preserve">Placa do concentrador RP2040 + Ethernet W5500 (W5500-EVB-Pico)</t>
   </si>
   <si>
-    <t xml:space="preserve">SparkFun DEV-19958 US$ 12,50 — 23/10/2026; convertido com câmbio × fator de importação</t>
+    <t xml:space="preserve">SparkFun DEV-19958 US$ 12,50, 23/10/2026; convertido com câmbio × fator de importação</t>
   </si>
   <si>
     <t xml:space="preserve">Cotado (US$)</t>
@@ -639,16 +639,16 @@
     <t xml:space="preserve">Fonte Mean Well LRS-150-12 (12 V / 12,5 A / 150 W)</t>
   </si>
   <si>
-    <t xml:space="preserve">MCEIG (fontesmeanwell.com.br) — 23/10/2026</t>
+    <t xml:space="preserve">MCEIG (fontesmeanwell.com.br), 23/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">P07</t>
   </si>
   <si>
-    <t xml:space="preserve">Fonte Mean Well LRS-150-5 (5 V / 26 A) — variante 5 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimativa (mesma família da LRS-150-12) — cotar</t>
+    <t xml:space="preserve">Fonte Mean Well LRS-150-5 (5 V / 26 A), variante 5 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimativa (mesma família da LRS-150-12), cotar</t>
   </si>
   <si>
     <t xml:space="preserve">P08</t>
@@ -657,7 +657,7 @@
     <t xml:space="preserve">Regulador step-down 12 V → 5 V (mini, 3 A)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa de mercado — cotar</t>
+    <t xml:space="preserve">Estimativa de mercado, cotar</t>
   </si>
   <si>
     <t xml:space="preserve">P09</t>
@@ -678,7 +678,7 @@
     <t xml:space="preserve">Plug RJ45 Cat5e (macho)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa (pote com 100) — cotar</t>
+    <t xml:space="preserve">Estimativa (pote com 100), cotar</t>
   </si>
   <si>
     <t xml:space="preserve">P12</t>
@@ -687,7 +687,7 @@
     <t xml:space="preserve">Cabo Cat5e (por metro)</t>
   </si>
   <si>
-    <t xml:space="preserve">KaBuM — Cabo Cat5e Fortrek FK500C 305 m R$ 1.229,41 (Pix) — 23/10/2026</t>
+    <t xml:space="preserve">KaBuM, Cabo Cat5e Fortrek FK500C 305 m R$ 1.229,41 (Pix), 23/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">P13</t>
@@ -714,7 +714,7 @@
     <t xml:space="preserve">Gabinete do concentrador ventilado (caixa IP54 + cooler 40 mm 12 V + filtro)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa — cotar (ambiente com poeira e calor)</t>
+    <t xml:space="preserve">Estimativa, cotar (ambiente com poeira e calor)</t>
   </si>
   <si>
     <t xml:space="preserve">P17</t>
@@ -732,7 +732,7 @@
     <t xml:space="preserve">Canaleta / perfil de fixação dos módulos (por metro)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa (canaleta PVC 20×10 mm em barra de 2 m) — cotar</t>
+    <t xml:space="preserve">Estimativa (canaleta PVC 20×10 mm em barra de 2 m), cotar</t>
   </si>
   <si>
     <t xml:space="preserve">P19</t>
@@ -747,13 +747,13 @@
     <t xml:space="preserve">Switch 24 portas Gigabit TP-Link TL-SG1024DE</t>
   </si>
   <si>
-    <t xml:space="preserve">KaBuM — 23/10/2026 (Pix)</t>
+    <t xml:space="preserve">KaBuM, 23/10/2026 (Pix)</t>
   </si>
   <si>
     <t xml:space="preserve">P21</t>
   </si>
   <si>
-    <t xml:space="preserve">Fita LED endereçável WS2812 — guia de coluna (por LED) [opcional]</t>
+    <t xml:space="preserve">Fita LED endereçável WS2812, guia de coluna (por LED) [opcional]</t>
   </si>
   <si>
     <t xml:space="preserve">LED</t>
@@ -765,7 +765,7 @@
     <t xml:space="preserve">Tag NFC NTAG213 adesiva 13,56 MHz</t>
   </si>
   <si>
-    <t xml:space="preserve">Loja RFID — lote 100 un R$ 237,41 à vista — 23/10/2026</t>
+    <t xml:space="preserve">Loja RFID, lote 100 un R$ 237,41 à vista, 23/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">P23</t>
@@ -780,7 +780,7 @@
     <t xml:space="preserve">ESP32-C3 Super Mini (pulseira)</t>
   </si>
   <si>
-    <t xml:space="preserve">Usinainfo — 23/10/2026 (Pix)</t>
+    <t xml:space="preserve">Usinainfo, 23/10/2026 (Pix)</t>
   </si>
   <si>
     <t xml:space="preserve">P25</t>
@@ -789,7 +789,7 @@
     <t xml:space="preserve">Módulo leitor NFC PN532 (43×40 mm, com cartão e chaveiro)</t>
   </si>
   <si>
-    <t xml:space="preserve">MakerHero — Kit Módulo Leitor RFID NFC PN532 — 23/10/2026 (Pix)</t>
+    <t xml:space="preserve">MakerHero, Kit Módulo Leitor RFID NFC PN532, 23/10/2026 (Pix)</t>
   </si>
   <si>
     <t xml:space="preserve">P26</t>
@@ -807,7 +807,7 @@
     <t xml:space="preserve">P28</t>
   </si>
   <si>
-    <t xml:space="preserve">Display LCD 20×4 I2C (painel da estação — Arq. B2)</t>
+    <t xml:space="preserve">Display LCD 20×4 I2C (painel da estação, Arq. B2)</t>
   </si>
   <si>
     <t xml:space="preserve">P29</t>
@@ -816,7 +816,7 @@
     <t xml:space="preserve">Módulo PTL comercial 3 dígitos + botão (RS-485)</t>
   </si>
   <si>
-    <t xml:space="preserve">Alibaba — Sophia T-P3: US$ 32 (1-299 un) / US$ 28 (300+) — 23/10/2026; média US$ 30</t>
+    <t xml:space="preserve">Alibaba, Sophia T-P3: US$ 32 (1-299 un) / US$ 28 (300+), 23/10/2026; média US$ 30</t>
   </si>
   <si>
     <t xml:space="preserve">P30</t>
@@ -825,7 +825,7 @@
     <t xml:space="preserve">Módulo PTL comercial endereço + quantidade (display alfanumérico)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa (não há preço público) — solicitar cotação a fornecedores</t>
+    <t xml:space="preserve">Estimativa (não há preço público), solicitar cotação a fornecedores</t>
   </si>
   <si>
     <t xml:space="preserve">P31</t>
@@ -834,13 +834,13 @@
     <t xml:space="preserve">Controlador/gateway PTL comercial por estação</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa (não há preço público) — solicitar cotação</t>
+    <t xml:space="preserve">Estimativa (não há preço público), solicitar cotação</t>
   </si>
   <si>
     <t xml:space="preserve">P32</t>
   </si>
   <si>
-    <t xml:space="preserve">PCB própria montada por EMS — Módulo Q (MCU + display 0,56" + botão + 2× RJ45)</t>
+    <t xml:space="preserve">PCB própria montada por EMS, Módulo Q (MCU + display 0,56" + botão + 2× RJ45)</t>
   </si>
   <si>
     <t xml:space="preserve">Estimativa com base na tabela de montagem JLCPCB (jlcpcb.com/help/article/pcb-assembly-price) + componentes</t>
@@ -849,7 +849,7 @@
     <t xml:space="preserve">P33</t>
   </si>
   <si>
-    <t xml:space="preserve">PCB própria montada por EMS — Módulo E+Q</t>
+    <t xml:space="preserve">PCB própria montada por EMS, Módulo E+Q</t>
   </si>
   <si>
     <t xml:space="preserve">Estimativa (idem)</t>
@@ -858,7 +858,7 @@
     <t xml:space="preserve">P34</t>
   </si>
   <si>
-    <t xml:space="preserve">PCB própria montada por EMS — Concentrador (MCU + Ethernet + 2× RS-485)</t>
+    <t xml:space="preserve">PCB própria montada por EMS, Concentrador (MCU + Ethernet + 2× RS-485)</t>
   </si>
   <si>
     <t xml:space="preserve">P35</t>
@@ -870,25 +870,25 @@
     <t xml:space="preserve">projeto</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimativa — solicitar orçamento a design house</t>
+    <t xml:space="preserve">Estimativa, solicitar orçamento a design house</t>
   </si>
   <si>
     <t xml:space="preserve">P36</t>
   </si>
   <si>
-    <t xml:space="preserve">Leitor RFID UHF de pulso comercial (FEIG HyWEAR Compact) — referência</t>
-  </si>
-  <si>
-    <t xml:space="preserve">atlasRFIDstore — US$ 997 — 22/10/2026 (UHF; não lê tags NFC)</t>
+    <t xml:space="preserve">Leitor RFID UHF de pulso comercial (FEIG HyWEAR Compact), referência</t>
+  </si>
+  <si>
+    <t xml:space="preserve">atlasRFIDstore, US$ 997, 22/10/2026 (UHF; não lê tags NFC)</t>
   </si>
   <si>
     <t xml:space="preserve">P37</t>
   </si>
   <si>
-    <t xml:space="preserve">Leitor HF/NFC fixo industrial (USB/RS-232) — alternativa comercial ao PN532</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimativa — cotar (ex.: ACS ACR122U ou similar)</t>
+    <t xml:space="preserve">Leitor HF/NFC fixo industrial (USB/RS-232), alternativa comercial ao PN532</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimativa, cotar (ex.: ACS ACR122U ou similar)</t>
   </si>
   <si>
     <t xml:space="preserve">Conjunto</t>
@@ -906,49 +906,49 @@
     <t xml:space="preserve">Módulo Q</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Módulo Q</t>
+    <t xml:space="preserve">Custo unitário, Módulo Q</t>
   </si>
   <si>
     <t xml:space="preserve">Nó de coluna</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Nó de coluna</t>
+    <t xml:space="preserve">Custo unitário, Nó de coluna</t>
   </si>
   <si>
     <t xml:space="preserve">Módulo E+Q</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Módulo E+Q</t>
+    <t xml:space="preserve">Custo unitário, Módulo E+Q</t>
   </si>
   <si>
     <t xml:space="preserve">Concentrador 12 V</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Concentrador 12 V</t>
+    <t xml:space="preserve">Custo unitário, Concentrador 12 V</t>
   </si>
   <si>
     <t xml:space="preserve">Concentrador 5 V</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Concentrador 5 V</t>
+    <t xml:space="preserve">Custo unitário, Concentrador 5 V</t>
   </si>
   <si>
     <t xml:space="preserve">Pulseira RFID (B1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Pulseira RFID (B1)</t>
+    <t xml:space="preserve">Custo unitário, Pulseira RFID (B1)</t>
   </si>
   <si>
     <t xml:space="preserve">Leitor fixo + painel (B2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Leitor fixo + painel (B2)</t>
+    <t xml:space="preserve">Custo unitário, Leitor fixo + painel (B2)</t>
   </si>
   <si>
     <t xml:space="preserve">Tag por caixa (B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo unitário — Tag por caixa (B)</t>
+    <t xml:space="preserve">Custo unitário, Tag por caixa (B)</t>
   </si>
   <si>
     <t xml:space="preserve">Variante 5 V: os módulos e nós não usam regulador step-down (P08); o custo é descontado na aba A-Interno.</t>
@@ -969,7 +969,7 @@
     <t xml:space="preserve">Total completo (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Arquitetura A — produção e montagem interna (12 V)</t>
+    <t xml:space="preserve">Arquitetura A, produção e montagem interna (12 V)</t>
   </si>
   <si>
     <t xml:space="preserve">Módulos Q (alto giro 0-3)</t>
@@ -1029,7 +1029,7 @@
     <t xml:space="preserve">estações ÷ portas por switch (arredondado para cima)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUBTOTAL PEÇAS — Arquitetura A (12 V)</t>
+    <t xml:space="preserve">SUBTOTAL PEÇAS, Arquitetura A (12 V)</t>
   </si>
   <si>
     <t xml:space="preserve">Mão de obra interna</t>
@@ -1068,7 +1068,7 @@
     <t xml:space="preserve">SUBTOTAL MÃO DE OBRA</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL — Arquitetura A interna (peças + mão de obra)</t>
+    <t xml:space="preserve">TOTAL, Arquitetura A interna (peças + mão de obra)</t>
   </si>
   <si>
     <t xml:space="preserve">Variante 5 V (peças)</t>
@@ -1089,10 +1089,10 @@
     <t xml:space="preserve">(+) Cabo de força extra para injeção de 5 V (m)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUBTOTAL PEÇAS — variante 5 V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opcional — guia de coluna no baixo giro (1 LED por prédio do fundo)</t>
+    <t xml:space="preserve">SUBTOTAL PEÇAS, variante 5 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opcional, guia de coluna no baixo giro (1 LED por prédio do fundo)</t>
   </si>
   <si>
     <t xml:space="preserve">LEDs guia de coluna</t>
@@ -1101,16 +1101,16 @@
     <t xml:space="preserve">prédios do fundo × (1 + reserva)</t>
   </si>
   <si>
-    <t xml:space="preserve">T1 — Placas próprias fabricadas e montadas por EMS (cada módulo com seu microcontrolador)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Módulo Q — PCB montada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Módulo E+Q — PCB montada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concentrador — PCB montada + fonte + gabinete</t>
+    <t xml:space="preserve">T1, Placas próprias fabricadas e montadas por EMS (cada módulo com seu microcontrolador)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulo Q, PCB montada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulo E+Q, PCB montada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentrador, PCB montada + fonte + gabinete</t>
   </si>
   <si>
     <t xml:space="preserve">estações × (1 + reserva)</t>
@@ -1140,10 +1140,10 @@
     <t xml:space="preserve">estações × (h instalação + h testes)</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL T1 — PCB própria (EMS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T2 — Sistema PTL comercial importado (hardware pronto; software de integração continua interno)</t>
+    <t xml:space="preserve">TOTAL T1, PCB própria (EMS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T2, Sistema PTL comercial importado (hardware pronto; software de integração continua interno)</t>
   </si>
   <si>
     <t xml:space="preserve">Módulos PTL 3 dígitos (alto giro 0-3)</t>
@@ -1164,7 +1164,7 @@
     <t xml:space="preserve">módulos em cadeia</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL T2 — PTL comercial importado</t>
+    <t xml:space="preserve">TOTAL T2, PTL comercial importado</t>
   </si>
   <si>
     <t xml:space="preserve">Valores em US$ convertidos por câmbio × fator de importação (aba Premissas). Itens de PTL comercial sem preço público devem ser cotados com fornecedores (ex.: ATOP, Aioi, fornecedores nacionais).</t>
@@ -1173,7 +1173,7 @@
     <t xml:space="preserve">Arquitetura B = infraestrutura de displays da Arquitetura A + identificação da caixa por RFID</t>
   </si>
   <si>
-    <t xml:space="preserve">Infraestrutura de displays (Arquitetura A interna — peças + mão de obra)</t>
+    <t xml:space="preserve">Infraestrutura de displays (Arquitetura A interna, peças + mão de obra)</t>
   </si>
   <si>
     <t xml:space="preserve">aba A-Interno</t>
@@ -1191,7 +1191,7 @@
     <t xml:space="preserve">30 s por caixa</t>
   </si>
   <si>
-    <t xml:space="preserve">B1 — Pulseira NFC (montagem própria)</t>
+    <t xml:space="preserve">B1, Pulseira NFC (montagem própria)</t>
   </si>
   <si>
     <t xml:space="preserve">Pulseiras NFC (ESP32-C3 + PN532 + bateria)</t>
@@ -1206,10 +1206,10 @@
     <t xml:space="preserve">1,5 h por pulseira</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL B1 — displays + tags + pulseiras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B2 — Leitor fixo na estação + painel (sem item no corpo do operador)</t>
+    <t xml:space="preserve">TOTAL B1, displays + tags + pulseiras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B2, Leitor fixo na estação + painel (sem item no corpo do operador)</t>
   </si>
   <si>
     <t xml:space="preserve">Leitor PN532 + LCD 20×4 + botão Fechar</t>
@@ -1224,13 +1224,13 @@
     <t xml:space="preserve">2 h por estação</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL B2 — displays + tags + leitor fixo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referência de mercado — leitor de pulso comercial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FEIG HyWEAR (UHF) por operador — não lê NFC; exigiria tags UHF</t>
+    <t xml:space="preserve">TOTAL B2, displays + tags + leitor fixo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referência de mercado, leitor de pulso comercial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FEIG HyWEAR (UHF) por operador, não lê NFC; exigiria tags UHF</t>
   </si>
   <si>
     <t xml:space="preserve">Coletores MovFast já existentes não entram no custo (Arquitetura A). Na Arquitetura B eles deixam de ser necessários na separação, mas continuam disponíveis para as demais operações.</t>
@@ -1272,7 +1272,7 @@
     <t xml:space="preserve">Consulta da caixa e, se possível, liberação para a próxima estação</t>
   </si>
   <si>
-    <t xml:space="preserve">App coletor Android (A1 — app próprio)</t>
+    <t xml:space="preserve">App coletor Android (A1, app próprio)</t>
   </si>
   <si>
     <t xml:space="preserve">A</t>
@@ -1326,13 +1326,13 @@
     <t xml:space="preserve">Operação, manutenção e suporte</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL — Arquitetura A com app próprio (sem tela WMS e sem itens só da B)</t>
+    <t xml:space="preserve">TOTAL, Arquitetura A com app próprio (sem tela WMS e sem itens só da B)</t>
   </si>
   <si>
     <t xml:space="preserve">Com a tela no WMS (A2) no lugar do app, troque 160 h por 80 h.</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL — Arquitetura B</t>
+    <t xml:space="preserve">TOTAL, Arquitetura B</t>
   </si>
 </sst>
 </file>
@@ -2065,7 +2065,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
         <v>23</v>
       </c>
@@ -5741,7 +5741,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
         <v>258</v>
       </c>
@@ -6006,7 +6006,7 @@
       </c>
       <c r="C2" s="32" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B2,Preços!$A:$A,0))</f>
-        <v>Display 7 segmentos 4 dígitos TM1637 (usa 3 dígitos — quantidade)</v>
+        <v>Display 7 segmentos 4 dígitos TM1637 (usa 3 dígitos, quantidade)</v>
       </c>
       <c r="D2" s="14" t="n">
         <v>1</v>
@@ -6331,7 +6331,7 @@
       </c>
       <c r="C19" s="32" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B19,Preços!$A:$A,0))</f>
-        <v>Display 7 segmentos 4 dígitos TM1637 (usa 3 dígitos — quantidade)</v>
+        <v>Display 7 segmentos 4 dígitos TM1637 (usa 3 dígitos, quantidade)</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>1</v>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="C40" s="32" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B40,Preços!$A:$A,0))</f>
-        <v>Fonte Mean Well LRS-150-5 (5 V / 26 A) — variante 5 V</v>
+        <v>Fonte Mean Well LRS-150-5 (5 V / 26 A), variante 5 V</v>
       </c>
       <c r="D40" s="14" t="n">
         <v>1</v>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="C53" s="32" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B53,Preços!$A:$A,0))</f>
-        <v>Display LCD 20×4 I2C (painel da estação — Arq. B2)</v>
+        <v>Display LCD 20×4 I2C (painel da estação, Arq. B2)</v>
       </c>
       <c r="D53" s="14" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
POC das estações 04 e 27, caixas maiores e sem luzes no topo
- Aba POC no orçamento: fase 1 (bancada) e fase 2 (estações 04 e 27),
  contingência e horas de software da POC; piloto passa a ser 04 e 27
- Diagrama do mockup da bancada (bancada_poc.png)
- 3D: sem LED guia e sem produtos coloridos em cima das caixas; caixas
  ocupam a largura do vão
- LED guia de coluna retirado do orçamento, do documento e dos diagramas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TBWA3G7ku1j3oTf4VMkLud
</commit_message>
<xml_diff>
--- a/projeto/entregaveis/Orcamento_PTL.xlsx
+++ b/projeto/entregaveis/Orcamento_PTL.xlsx
@@ -18,6 +18,7 @@
     <sheet name="A-Terceiros" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="B-RFID" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Software" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="POC" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="614">
   <si>
     <t xml:space="preserve">Orçamento do projeto Pick-to-Light (flow rack)</t>
   </si>
@@ -49,7 +50,7 @@
     <t xml:space="preserve">• Aba 'Estações': números de endereços por estação, extraídos de wms_endereco (esteiras 1 e 2) em 23/10/2026. Corrija qualquer número direto ali: todo o orçamento recalcula.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Coluna 'Piloto' (S/N) na aba 'Estações' define quais estações entram no cenário piloto (padrão: 05 e 27).</t>
+    <t xml:space="preserve">• Coluna 'Piloto' (S/N) na aba 'Estações' define quais estações entram no cenário piloto (POC: 04 e 27).</t>
   </si>
   <si>
     <t xml:space="preserve">• Aba 'Preços': catálogo de peças com fonte e data. Itens marcados 'Estimativa' devem ser cotados antes da compra.</t>
@@ -154,7 +155,7 @@
     <t xml:space="preserve">Resumo do orçamento, Pick-to-Light</t>
   </si>
   <si>
-    <t xml:space="preserve">Piloto: estações marcadas 'S' na aba Estações (padrão 05 e 27). A operação completa já inclui o piloto. Hardware, instalação e treinamento; software nas linhas abaixo.</t>
+    <t xml:space="preserve">Piloto: estações marcadas 'S' na aba Estações (POC: 04 e 27). A operação completa já inclui o piloto. Hardware, instalação e treinamento; software nas linhas abaixo.</t>
   </si>
   <si>
     <t xml:space="preserve">Cenário</t>
@@ -217,12 +218,6 @@
     <t xml:space="preserve">Displays (A interno) + tags + leitor fixo e painel (opção indicada na B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Opcional, guia de coluna no baixo giro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 LED por prédio do baixo giro</t>
-  </si>
-  <si>
     <t xml:space="preserve">Desenvolvimento de software (interno)</t>
   </si>
   <si>
@@ -242,6 +237,12 @@
   </si>
   <si>
     <t xml:space="preserve">B2 com contingência + software da Arquitetura B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POC (bancada + estações 04 e 27)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware com contingência (aba POC); software da POC é interno</t>
   </si>
   <si>
     <t xml:space="preserve">Volume da operação (informado): ~3.000 volumes/dia e 250.000 a 270.000 produtos separados por dia.</t>
@@ -617,12 +618,12 @@
     <t xml:space="preserve">Comum</t>
   </si>
   <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
     <t xml:space="preserve">05</t>
   </si>
   <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
     <t xml:space="preserve">06</t>
   </si>
   <si>
@@ -830,7 +831,7 @@
     <t xml:space="preserve">Fonte Mean Well LRS-150-12 (12 V / 12,5 A / 150 W)</t>
   </si>
   <si>
-    <t xml:space="preserve">MCEIG (fontesmeanwell.com.br), 23/10/2026. Carga estimada &lt; 40 W por estação: folga para LED guia e expansão</t>
+    <t xml:space="preserve">MCEIG (fontesmeanwell.com.br), 23/10/2026. Carga estimada &lt; 40 W por estação: folga para expansão</t>
   </si>
   <si>
     <t xml:space="preserve">P07</t>
@@ -950,12 +951,18 @@
     <t xml:space="preserve">P21</t>
   </si>
   <si>
-    <t xml:space="preserve">Fita LED endereçável WS2812, guia de coluna (por LED) [opcional]</t>
+    <t xml:space="preserve">(não usado) LED guia de coluna, retirado em 26/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">LED</t>
   </si>
   <si>
+    <t xml:space="preserve">Não faz parte do projeto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retirado</t>
+  </si>
+  <si>
     <t xml:space="preserve">P22</t>
   </si>
   <si>
@@ -1157,6 +1164,21 @@
     <t xml:space="preserve">Estimativa, cotar com a manutenção predial</t>
   </si>
   <si>
+    <t xml:space="preserve">P48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painel de MDF 1,2 × 0,6 m com longarina para a bancada + parafusos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switch 5 portas (bancada)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimativa, cotar (ou porta livre de switch existente)</t>
+  </si>
+  <si>
     <t xml:space="preserve">P47</t>
   </si>
   <si>
@@ -1430,15 +1452,6 @@
     <t xml:space="preserve">SUBTOTAL MATERIAIS, variante 5 V</t>
   </si>
   <si>
-    <t xml:space="preserve">Opcional, guia de coluna no baixo giro (1 LED por prédio do baixo giro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEDs guia de coluna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prédios do baixo giro × (1 + reserva); ligados ao E+Q da zona</t>
-  </si>
-  <si>
     <t xml:space="preserve">T1, Placas próprias fabricadas e montadas por EMS (cada módulo com seu microcontrolador)</t>
   </si>
   <si>
@@ -1682,7 +1695,7 @@
     <t xml:space="preserve">Testes integrados, piloto e homologação</t>
   </si>
   <si>
-    <t xml:space="preserve">Inclui ajustes no piloto (estações 05 e 27)</t>
+    <t xml:space="preserve">Inclui ajustes na POC (estações 04 e 27)</t>
   </si>
   <si>
     <t xml:space="preserve">Documentação e treinamento</t>
@@ -1701,6 +1714,171 @@
   </si>
   <si>
     <t xml:space="preserve">Custo-hora de desenvolvimento calculado na aba Premissas (salário de mercado × encargos ÷ horas). É custo interno da equipe, não desembolso extra, a menos que o desenvolvimento seja contratado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POC: bancada + estações 04 e 27 (Arquitetura A, coletor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 1 valida o hardware e o software na bancada; fase 2 instala nas estações 04 (Medicamento) e 27 (Perfumaria). As estações da POC são as marcadas 'S' na aba Estações.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qtd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 1, bancada (1 coluna de alto giro, 1 zona de cada tipo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentrador 12 V completo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gabinete, fonte, placa, alimentação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 prédio de alto giro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulos Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 andares (0 a 3) do prédio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 zona dos andares 4-5 + 1 zona do baixo giro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barra âmbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabo Cat5e (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barramento e ligações da bancada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plugs RJ45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painel de MDF com longarina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">simula a prateleira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Switch 5 portas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rede da bancada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compra única, servem para a fase 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compra única, serve para a fase 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% sobre os itens acima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montagem dos módulos (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conc. + nó + 4 Q + 2 E+Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testes de bancada (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">acender, confirmar, falha, troca e cadastro de LED, 48 h de operação contínua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL FASE 1, bancada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 2, instalação nas estações 04 e 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiais, montagem, instalação e treinamento das 2 estações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aba A-Interno, coluna piloto (estações com 'S')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(−) Ferramentas já compradas na fase 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kit de rede + bancada de eletrônica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(−) Módulos da bancada reaproveitados na estação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">o concentrador, o nó, os 4 Q e os 2 E+Q da bancada vão para a estação 04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL FASE 2, estações 04 e 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HARDWARE DA POC (fase 1 + fase 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingência</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% sobre o hardware da POC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HARDWARE DA POC COM CONTINGÊNCIA (desembolso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software para a POC (equipe interna, versão mínima)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firmware do concentrador, dos nós e dos E+Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barramento, endereçamento, diagnóstico, cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serviço PTL, versão mínima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abrir e fechar caixa, acender, confirmar, sinal de baixo giro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integração Sybase (leitura dos itens da caixa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">views de leitura e gravação de eventos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App do coletor (A1), versão mínima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leitura com gatilho e progresso da caixa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interface de controle, versão mínima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">falhas de LED e cadastro por endereço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testes da bancada e operação assistida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ajustes durante a POC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOFTWARE DA POC (horas e custo interno)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prazo estimado: bancada 3 a 4 semanas; instalação nas 2 estações 1 semana; operação assistida 4 semanas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O software da POC é a primeira parte do software do projeto (aba Software), não um custo a mais.</t>
   </si>
 </sst>
 </file>
@@ -1873,7 +2051,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2043,6 +2221,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2545,27 +2727,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C2" s="20" t="n">
         <v>240</v>
@@ -2575,15 +2757,15 @@
         <v>24907.8773006135</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C3" s="20" t="n">
         <v>120</v>
@@ -2593,15 +2775,15 @@
         <v>12453.9386503067</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>526</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>522</v>
       </c>
       <c r="C4" s="20" t="n">
         <v>60</v>
@@ -2611,15 +2793,15 @@
         <v>6226.96932515337</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="C5" s="20" t="n">
         <v>160</v>
@@ -2629,15 +2811,15 @@
         <v>16605.2515337423</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="C6" s="20" t="n">
         <v>80</v>
@@ -2647,15 +2829,15 @@
         <v>8302.62576687117</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C7" s="20" t="n">
         <v>120</v>
@@ -2665,15 +2847,15 @@
         <v>12453.9386503067</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C8" s="20" t="n">
         <v>100</v>
@@ -2683,15 +2865,15 @@
         <v>10378.282208589</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="C9" s="20" t="n">
         <v>80</v>
@@ -2701,15 +2883,15 @@
         <v>8302.62576687117</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C10" s="20" t="n">
         <v>120</v>
@@ -2719,15 +2901,15 @@
         <v>12453.9386503067</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C11" s="20" t="n">
         <v>40</v>
@@ -2737,15 +2919,15 @@
         <v>4151.31288343558</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C12" s="20" t="n">
         <v>24</v>
@@ -2755,15 +2937,15 @@
         <v>2490.78773006135</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C13" s="20" t="n">
         <v>120</v>
@@ -2773,15 +2955,15 @@
         <v>12453.9386503067</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C14" s="20" t="n">
         <v>40</v>
@@ -2791,12 +2973,12 @@
         <v>4151.31288343558</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="42" t="n">
@@ -2808,12 +2990,12 @@
         <v>118727.548466258</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="42" t="n">
@@ -2828,7 +3010,583 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>561</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>564</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>565</v>
+      </c>
+      <c r="C5" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="37" t="n">
+        <f aca="false">Composição!$F$39</f>
+        <v>549.810425</v>
+      </c>
+      <c r="E5" s="31" t="n">
+        <f aca="false">C5*D5</f>
+        <v>549.810425</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>388</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>566</v>
+      </c>
+      <c r="C6" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="37" t="n">
+        <f aca="false">Composição!$F$16</f>
+        <v>96.8</v>
+      </c>
+      <c r="E6" s="31" t="n">
+        <f aca="false">C6*D6</f>
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>568</v>
+      </c>
+      <c r="C7" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <f aca="false">Composição!$F$8</f>
+        <v>45.1417049180328</v>
+      </c>
+      <c r="E7" s="31" t="n">
+        <f aca="false">C7*D7</f>
+        <v>180.566819672131</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>569</v>
+      </c>
+      <c r="C8" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <f aca="false">Composição!$F$27</f>
+        <v>134.95</v>
+      </c>
+      <c r="E8" s="31" t="n">
+        <f aca="false">C8*D8</f>
+        <v>269.9</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="C9" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="37" t="n">
+        <f aca="false">Preços!$D$50</f>
+        <v>45</v>
+      </c>
+      <c r="E9" s="31" t="n">
+        <f aca="false">C9*D9</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>571</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>572</v>
+      </c>
+      <c r="C10" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="37" t="n">
+        <f aca="false">Preços!$D$13</f>
+        <v>4.03085245901639</v>
+      </c>
+      <c r="E10" s="31" t="n">
+        <f aca="false">C10*D10</f>
+        <v>80.6170491803279</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>573</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="37" t="n">
+        <f aca="false">Preços!$D$12</f>
+        <v>0.8</v>
+      </c>
+      <c r="E11" s="31" t="n">
+        <f aca="false">C11*D11</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>574</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>575</v>
+      </c>
+      <c r="C12" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="37" t="n">
+        <f aca="false">Preços!$D$48</f>
+        <v>150</v>
+      </c>
+      <c r="E12" s="31" t="n">
+        <f aca="false">C12*D12</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>577</v>
+      </c>
+      <c r="C13" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="37" t="n">
+        <f aca="false">Preços!$D$49</f>
+        <v>90</v>
+      </c>
+      <c r="E13" s="31" t="n">
+        <f aca="false">C13*D13</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="C14" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="37" t="n">
+        <f aca="false">Preços!$D$42</f>
+        <v>285.99</v>
+      </c>
+      <c r="E14" s="31" t="n">
+        <f aca="false">C14*D14</f>
+        <v>285.99</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>579</v>
+      </c>
+      <c r="C15" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="37" t="n">
+        <f aca="false">Preços!$D$43</f>
+        <v>700</v>
+      </c>
+      <c r="E15" s="31" t="n">
+        <f aca="false">C15*D15</f>
+        <v>700</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>443</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>580</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="40" t="n">
+        <f aca="false">Premissas!$B$27</f>
+        <v>0.05</v>
+      </c>
+      <c r="E16" s="31" t="n">
+        <f aca="false">D16*SUM(E5:E15)</f>
+        <v>123.234214692623</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>581</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>582</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <f aca="false">Premissas!$B$15+Premissas!$B$13+4*Premissas!$B$12+2*Premissas!$B$14</f>
+        <v>5.75</v>
+      </c>
+      <c r="D17" s="37" t="n">
+        <f aca="false">Premissas!$B$9</f>
+        <v>34.9305521472393</v>
+      </c>
+      <c r="E17" s="31" t="n">
+        <f aca="false">C17*D17</f>
+        <v>200.850674846626</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>583</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>584</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="D18" s="37" t="n">
+        <f aca="false">Premissas!$B$9</f>
+        <v>34.9305521472393</v>
+      </c>
+      <c r="E18" s="31" t="n">
+        <f aca="false">C18*D18</f>
+        <v>558.888834355828</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>585</v>
+      </c>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="38" t="n">
+        <f aca="false">SUM(E5:E18)</f>
+        <v>3347.65801774754</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>587</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>588</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="37" t="n">
+        <f aca="false">'A-Interno'!F34</f>
+        <v>19211.4974214212</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>589</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>590</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="31" t="n">
+        <f aca="false">-('A-Interno'!F18+'A-Interno'!F19)*(1+Premissas!$B$27)</f>
+        <v>-1035.2895</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>591</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>592</v>
+      </c>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="31" t="n">
+        <f aca="false">-(Composição!$F$39+Composição!$F$16+4*Composição!$F$8+2*Composição!$F$27)</f>
+        <v>-1097.07724467213</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
+        <v>593</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="38" t="n">
+        <f aca="false">SUM(E22:E24)</f>
+        <v>17079.1306767491</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
+        <v>594</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="38" t="n">
+        <f aca="false">E19+E25</f>
+        <v>20426.7886944966</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>595</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>596</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="40" t="n">
+        <f aca="false">Premissas!$B$28</f>
+        <v>0.1</v>
+      </c>
+      <c r="E28" s="31" t="n">
+        <f aca="false">D28*E27</f>
+        <v>2042.67886944966</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="38" t="n">
+        <f aca="false">E27+E28</f>
+        <v>22469.4675639463</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>599</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>600</v>
+      </c>
+      <c r="C32" s="20" t="n">
+        <v>160</v>
+      </c>
+      <c r="D32" s="37" t="n">
+        <f aca="false">Premissas!$B$10</f>
+        <v>103.78282208589</v>
+      </c>
+      <c r="E32" s="31" t="n">
+        <f aca="false">C32*D32</f>
+        <v>16605.2515337423</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>601</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="C33" s="20" t="n">
+        <v>160</v>
+      </c>
+      <c r="D33" s="37" t="n">
+        <f aca="false">Premissas!$B$10</f>
+        <v>103.78282208589</v>
+      </c>
+      <c r="E33" s="31" t="n">
+        <f aca="false">C33*D33</f>
+        <v>16605.2515337423</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>603</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>604</v>
+      </c>
+      <c r="C34" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="D34" s="37" t="n">
+        <f aca="false">Premissas!$B$10</f>
+        <v>103.78282208589</v>
+      </c>
+      <c r="E34" s="31" t="n">
+        <f aca="false">C34*D34</f>
+        <v>6226.96932515337</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>605</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="C35" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="D35" s="37" t="n">
+        <f aca="false">Premissas!$B$10</f>
+        <v>103.78282208589</v>
+      </c>
+      <c r="E35" s="31" t="n">
+        <f aca="false">C35*D35</f>
+        <v>10378.282208589</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>607</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>608</v>
+      </c>
+      <c r="C36" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="D36" s="37" t="n">
+        <f aca="false">Premissas!$B$10</f>
+        <v>103.78282208589</v>
+      </c>
+      <c r="E36" s="31" t="n">
+        <f aca="false">C36*D36</f>
+        <v>4151.31288343558</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>609</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>610</v>
+      </c>
+      <c r="C37" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="D37" s="37" t="n">
+        <f aca="false">Premissas!$B$10</f>
+        <v>103.78282208589</v>
+      </c>
+      <c r="E37" s="31" t="n">
+        <f aca="false">C37*D37</f>
+        <v>8302.62576687117</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>611</v>
+      </c>
+      <c r="B38" s="16"/>
+      <c r="C38" s="42" t="n">
+        <f aca="false">SUM(C32:C37)</f>
+        <v>600</v>
+      </c>
+      <c r="D38" s="16"/>
+      <c r="E38" s="38" t="n">
+        <f aca="false">SUM(E32:E37)</f>
+        <v>62269.6932515337</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="s">
+        <v>613</v>
       </c>
     </row>
   </sheetData>
@@ -2847,7 +3605,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -3055,59 +3813,50 @@
         <v>364675.901003489</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="9" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="10" t="n">
-        <f aca="false">'A-Interno'!F43</f>
-        <v>49.5</v>
-      </c>
-      <c r="D11" s="10" t="n">
-        <f aca="false">'A-Interno'!G43</f>
-        <v>1016.1</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <f aca="false">D11/Estações!$O$43</f>
-        <v>25.4025</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <f aca="false">D11*(1+Premissas!$B$28)</f>
-        <v>1117.71</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>64</v>
+      <c r="B13" s="13" t="str">
+        <f aca="false">"Horas: "&amp;TEXT(Software!C15,"#,##0")</f>
+        <v>Horas: 1,144</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <f aca="false">Software!D15</f>
+        <v>118727.548466258</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" s="13" t="str">
-        <f aca="false">"Horas: "&amp;TEXT(Software!C15,"#,##0")</f>
-        <v>Horas: 1,144</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <f aca="false">Software!D15</f>
-        <v>118727.548466258</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="13" t="str">
         <f aca="false">"Horas: "&amp;TEXT(Software!C16,"#,##0")</f>
         <v>Horas: 1,064</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D14" s="10" t="n">
         <f aca="false">Software!D16</f>
         <v>110424.922699387</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="17" t="n">
+        <f aca="false">F6+D13</f>
+        <v>453958.589699724</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3121,27 +3870,27 @@
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="17" t="n">
-        <f aca="false">F6+D14</f>
-        <v>453958.589699724</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+        <f aca="false">F10+D14</f>
+        <v>475100.823702875</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B19" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17" t="n">
-        <f aca="false">F10+D15</f>
-        <v>475100.823702875</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="C19" s="17" t="n">
+        <f aca="false">POC!E29</f>
+        <v>22469.4675639463</v>
+      </c>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>71</v>
       </c>
     </row>
@@ -3929,7 +4678,7 @@
         <v>192</v>
       </c>
       <c r="D3" s="24" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E3" s="25" t="n">
         <v>201</v>
@@ -3969,7 +4718,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>188</v>
@@ -3978,7 +4727,7 @@
         <v>192</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E4" s="25" t="n">
         <v>209</v>
@@ -4909,7 +5658,7 @@
         <v>192</v>
       </c>
       <c r="D23" s="24" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E23" s="25" t="n">
         <v>181</v>
@@ -5892,7 +6641,7 @@
       </c>
       <c r="E44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",E2:E41)</f>
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="F44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",F2:F41)</f>
@@ -5900,7 +6649,7 @@
       </c>
       <c r="G44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",G2:G41)</f>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",H2:H41)</f>
@@ -5908,7 +6657,7 @@
       </c>
       <c r="I44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",I2:I41)</f>
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="J44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",J2:J41)</f>
@@ -5920,7 +6669,7 @@
       </c>
       <c r="L44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",L2:L41)</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M44" s="29" t="n">
         <f aca="false">SUMIF($D$2:$D$41,"S",M2:M41)</f>
@@ -5972,7 +6721,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -6441,23 +7190,23 @@
       <c r="C22" s="13" t="s">
         <v>305</v>
       </c>
-      <c r="D22" s="33" t="n">
-        <v>0.9</v>
+      <c r="D22" s="30" t="n">
+        <v>0</v>
       </c>
       <c r="E22" s="13"/>
       <c r="F22" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="G22" s="34" t="s">
-        <v>107</v>
+        <v>306</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>165</v>
@@ -6467,7 +7216,7 @@
       </c>
       <c r="E23" s="13"/>
       <c r="F23" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>248</v>
@@ -6475,10 +7224,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>165</v>
@@ -6496,10 +7245,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>165</v>
@@ -6509,7 +7258,7 @@
       </c>
       <c r="E25" s="13"/>
       <c r="F25" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>248</v>
@@ -6517,10 +7266,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>165</v>
@@ -6530,7 +7279,7 @@
       </c>
       <c r="E26" s="13"/>
       <c r="F26" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="G26" s="13" t="s">
         <v>248</v>
@@ -6538,10 +7287,10 @@
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>294</v>
@@ -6559,10 +7308,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>165</v>
@@ -6580,10 +7329,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>165</v>
@@ -6601,10 +7350,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>165</v>
@@ -6617,7 +7366,7 @@
         <v>30</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>261</v>
@@ -6625,10 +7374,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>165</v>
@@ -6641,7 +7390,7 @@
         <v>65</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="G31" s="34" t="s">
         <v>107</v>
@@ -6649,10 +7398,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>165</v>
@@ -6665,7 +7414,7 @@
         <v>220</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="G32" s="34" t="s">
         <v>107</v>
@@ -6673,10 +7422,10 @@
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>165</v>
@@ -6689,7 +7438,7 @@
         <v>9</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="G33" s="34" t="s">
         <v>107</v>
@@ -6697,10 +7446,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>165</v>
@@ -6713,7 +7462,7 @@
         <v>22</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G34" s="34" t="s">
         <v>107</v>
@@ -6721,10 +7470,10 @@
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C35" s="13" t="s">
         <v>165</v>
@@ -6737,7 +7486,7 @@
         <v>35</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G35" s="34" t="s">
         <v>107</v>
@@ -6745,20 +7494,20 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D36" s="33" t="n">
         <v>15000</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="9" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="G36" s="34" t="s">
         <v>107</v>
@@ -6766,10 +7515,10 @@
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>165</v>
@@ -6782,7 +7531,7 @@
         <v>997</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>261</v>
@@ -6790,10 +7539,10 @@
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C38" s="13" t="s">
         <v>165</v>
@@ -6803,7 +7552,7 @@
       </c>
       <c r="E38" s="13"/>
       <c r="F38" s="9" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G38" s="34" t="s">
         <v>107</v>
@@ -6811,10 +7560,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C39" s="13" t="s">
         <v>137</v>
@@ -6825,7 +7574,7 @@
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="9" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>248</v>
@@ -6833,10 +7582,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C40" s="13" t="s">
         <v>165</v>
@@ -6854,10 +7603,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C41" s="13" t="s">
         <v>165</v>
@@ -6875,10 +7624,10 @@
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C42" s="13" t="s">
         <v>294</v>
@@ -6888,7 +7637,7 @@
       </c>
       <c r="E42" s="13"/>
       <c r="F42" s="9" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G42" s="13" t="s">
         <v>248</v>
@@ -6896,10 +7645,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>294</v>
@@ -6917,10 +7666,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C44" s="13" t="s">
         <v>165</v>
@@ -6930,7 +7679,7 @@
       </c>
       <c r="E44" s="13"/>
       <c r="F44" s="9" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="G44" s="13" t="s">
         <v>248</v>
@@ -6938,10 +7687,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>294</v>
@@ -6951,7 +7700,7 @@
       </c>
       <c r="E45" s="13"/>
       <c r="F45" s="9" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="G45" s="34" t="s">
         <v>107</v>
@@ -6959,10 +7708,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>165</v>
@@ -6980,10 +7729,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C47" s="13" t="s">
         <v>165</v>
@@ -6993,7 +7742,7 @@
       </c>
       <c r="E47" s="13"/>
       <c r="F47" s="9" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="G47" s="34" t="s">
         <v>107</v>
@@ -7001,22 +7750,64 @@
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>165</v>
+        <v>294</v>
       </c>
       <c r="D48" s="33" t="n">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="E48" s="13"/>
       <c r="F48" s="9" t="s">
         <v>276</v>
       </c>
       <c r="G48" s="34" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D49" s="33" t="n">
+        <v>90</v>
+      </c>
+      <c r="E49" s="13"/>
+      <c r="F49" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="G49" s="34" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D50" s="33" t="n">
+        <v>45</v>
+      </c>
+      <c r="E50" s="13"/>
+      <c r="F50" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="G50" s="34" t="s">
         <v>107</v>
       </c>
     </row>
@@ -7048,7 +7839,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>239</v>
@@ -7057,18 +7848,18 @@
         <v>240</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>245</v>
@@ -7091,7 +7882,7 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>271</v>
@@ -7114,7 +7905,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>283</v>
@@ -7137,7 +7928,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>274</v>
@@ -7160,7 +7951,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>280</v>
@@ -7183,7 +7974,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>277</v>
@@ -7206,7 +7997,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -7219,7 +8010,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>252</v>
@@ -7242,7 +8033,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>255</v>
@@ -7265,7 +8056,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>268</v>
@@ -7288,7 +8079,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>287</v>
@@ -7311,7 +8102,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>274</v>
@@ -7334,7 +8125,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>285</v>
@@ -7357,7 +8148,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
@@ -7370,7 +8161,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>249</v>
@@ -7393,7 +8184,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>245</v>
@@ -7416,7 +8207,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>252</v>
@@ -7439,7 +8230,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>255</v>
@@ -7462,7 +8253,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B22" s="13" t="s">
         <v>268</v>
@@ -7485,7 +8276,7 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B23" s="13" t="s">
         <v>271</v>
@@ -7508,7 +8299,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B24" s="13" t="s">
         <v>274</v>
@@ -7531,7 +8322,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>285</v>
@@ -7554,7 +8345,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="B26" s="13" t="s">
         <v>287</v>
@@ -7577,7 +8368,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
@@ -7590,7 +8381,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B29" s="13" t="s">
         <v>258</v>
@@ -7613,7 +8404,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B30" s="13" t="s">
         <v>255</v>
@@ -7636,7 +8427,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B31" s="13" t="s">
         <v>262</v>
@@ -7659,7 +8450,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B32" s="13" t="s">
         <v>268</v>
@@ -7682,7 +8473,7 @@
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B33" s="13" t="s">
         <v>289</v>
@@ -7705,7 +8496,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B34" s="13" t="s">
         <v>292</v>
@@ -7728,7 +8519,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B35" s="13" t="s">
         <v>274</v>
@@ -7751,10 +8542,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C36" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B36,Preços!$A:$A,0))</f>
@@ -7774,10 +8565,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C37" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B37,Preços!$A:$A,0))</f>
@@ -7797,10 +8588,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C38" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B38,Preços!$A:$A,0))</f>
@@ -7820,7 +8611,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="16"/>
@@ -7833,7 +8624,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B41" s="13" t="s">
         <v>258</v>
@@ -7856,7 +8647,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B42" s="13" t="s">
         <v>255</v>
@@ -7879,7 +8670,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B43" s="13" t="s">
         <v>265</v>
@@ -7902,7 +8693,7 @@
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B44" s="13" t="s">
         <v>289</v>
@@ -7925,7 +8716,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B45" s="13" t="s">
         <v>292</v>
@@ -7948,7 +8739,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B46" s="13" t="s">
         <v>274</v>
@@ -7971,10 +8762,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C47" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B47,Preços!$A:$A,0))</f>
@@ -7994,10 +8785,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C48" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B48,Preços!$A:$A,0))</f>
@@ -8017,10 +8808,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C49" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B49,Preços!$A:$A,0))</f>
@@ -8040,7 +8831,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="16"/>
@@ -8053,10 +8844,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C52" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B52,Preços!$A:$A,0))</f>
@@ -8076,10 +8867,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C53" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B53,Preços!$A:$A,0))</f>
@@ -8099,10 +8890,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C54" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B54,Preços!$A:$A,0))</f>
@@ -8122,10 +8913,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="13" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C55" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B55,Preços!$A:$A,0))</f>
@@ -8145,7 +8936,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
@@ -8158,10 +8949,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C58" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B58,Preços!$A:$A,0))</f>
@@ -8181,10 +8972,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C59" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B59,Preços!$A:$A,0))</f>
@@ -8204,7 +8995,7 @@
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B60" s="13" t="s">
         <v>271</v>
@@ -8227,7 +9018,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B61" s="13" t="s">
         <v>252</v>
@@ -8250,7 +9041,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B62" s="13" t="s">
         <v>255</v>
@@ -8273,7 +9064,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B63" s="13" t="s">
         <v>268</v>
@@ -8296,7 +9087,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B64" s="13" t="s">
         <v>287</v>
@@ -8319,7 +9110,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B65" s="13" t="s">
         <v>274</v>
@@ -8342,7 +9133,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B66" s="13" t="s">
         <v>285</v>
@@ -8365,7 +9156,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B67" s="13" t="s">
         <v>280</v>
@@ -8388,7 +9179,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="13" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B68" s="13" t="s">
         <v>277</v>
@@ -8411,7 +9202,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B69" s="16"/>
       <c r="C69" s="16"/>
@@ -8424,10 +9215,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="13" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C71" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B71,Preços!$A:$A,0))</f>
@@ -8447,10 +9238,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C72" s="36" t="str">
         <f aca="false">INDEX(Preços!$B:$B,MATCH(B72,Preços!$A:$A,0))</f>
@@ -8470,7 +9261,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="B73" s="16"/>
       <c r="C73" s="16"/>
@@ -8483,17 +9274,17 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -8512,7 +9303,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -8529,35 +9320,35 @@
         <v>240</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="C3" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$F$44*(1+Premissas!$B$26),0)</f>
@@ -8582,10 +9373,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C4" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$K$44*(1+Premissas!$B$26),0)</f>
@@ -8610,10 +9401,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C5" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$26),0)</f>
@@ -8638,10 +9429,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="C6" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$O$44*(1+Premissas!$B$26),0)</f>
@@ -8666,10 +9457,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="C7" s="39" t="n">
         <f aca="false">Estações!$N$44*Premissas!$B$29+Estações!$O$44*2*Premissas!$B$30</f>
@@ -8694,10 +9485,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="C8" s="39" t="n">
         <f aca="false">Estações!$N$44*2+Estações!$O$44*4</f>
@@ -8722,10 +9513,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="C9" s="39" t="n">
         <f aca="false">Estações!$K$44*(Premissas!$B$31*Premissas!$B$32+Premissas!$B$33)+Estações!$O$44*2*Premissas!$B$34+Estações!$O$44*Premissas!$B$35</f>
@@ -8750,10 +9541,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="C10" s="39" t="n">
         <f aca="false">Estações!$O$44</f>
@@ -8778,10 +9569,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="C11" s="39" t="n">
         <f aca="false">Estações!$O$44</f>
@@ -8792,7 +9583,7 @@
         <v>40</v>
       </c>
       <c r="E11" s="37" t="n">
-        <f aca="false">Preços!$D$48</f>
+        <f aca="false">Preços!$D$50</f>
         <v>45</v>
       </c>
       <c r="F11" s="31" t="n">
@@ -8806,10 +9597,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="C12" s="39" t="n">
         <f aca="false">Estações!$O$44*Premissas!$B$36</f>
@@ -8834,10 +9625,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="C13" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$O$44/Premissas!$B$37,0)</f>
@@ -8862,10 +9653,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C14" s="39" t="n">
         <f aca="false">C13</f>
@@ -8890,10 +9681,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C15" s="39" t="n">
         <f aca="false">C13</f>
@@ -8918,10 +9709,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="C16" s="39" t="n">
         <f aca="false">C13*Premissas!$B$38</f>
@@ -8946,10 +9737,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="C17" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$O$44*Premissas!$B$39,0)</f>
@@ -8974,10 +9765,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C18" s="39" t="n">
         <f aca="false">1</f>
@@ -9002,10 +9793,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C19" s="39" t="n">
         <f aca="false">1</f>
@@ -9030,10 +9821,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -9052,7 +9843,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
@@ -9069,15 +9860,15 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">C3*Premissas!$B$12</f>
@@ -9102,10 +9893,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="C25" s="21" t="n">
         <f aca="false">C4*Premissas!$B$13</f>
@@ -9130,10 +9921,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="C26" s="21" t="n">
         <f aca="false">C5*Premissas!$B$14</f>
@@ -9158,10 +9949,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="C27" s="21" t="n">
         <f aca="false">C6*Premissas!$B$15</f>
@@ -9186,10 +9977,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="C28" s="21" t="n">
         <f aca="false">(Estações!$O$44*Premissas!$B$16+Estações!$F$44*Premissas!$B$17+Estações!$K$44*Premissas!$B$18+Estações!$M$44*Premissas!$B$19+C9*Premissas!$B$20)*Premissas!$B$22</f>
@@ -9214,10 +10005,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="C29" s="21" t="n">
         <f aca="false">Estações!$O$44*Premissas!$B$21*Premissas!$B$22</f>
@@ -9242,10 +10033,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">Estações!$O$44*Premissas!$B$23*Premissas!$B$24</f>
@@ -9270,10 +10061,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">Premissas!$B$25</f>
@@ -9298,7 +10089,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="41" t="n">
@@ -9321,7 +10112,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
@@ -9338,15 +10129,15 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="C37" s="39" t="n">
         <f aca="false">-(C4+C5+C6)</f>
@@ -9371,10 +10162,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="C38" s="39" t="n">
         <f aca="false">C6</f>
@@ -9399,10 +10190,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="C39" s="39" t="n">
         <f aca="false">Estações!$O$44*Premissas!$B$42</f>
@@ -9427,7 +10218,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="B40" s="16"/>
       <c r="C40" s="16"/>
@@ -9440,39 +10231,6 @@
       <c r="G40" s="38" t="n">
         <f aca="false">G21+SUM(G37:G39)</f>
         <v>227135.487797295</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="s">
-        <v>465</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>466</v>
-      </c>
-      <c r="C43" s="39" t="n">
-        <f aca="false">ROUNDUP(Estações!$L$44*(1+Premissas!$B$26),0)</f>
-        <v>55</v>
-      </c>
-      <c r="D43" s="39" t="n">
-        <f aca="false">ROUNDUP(Estações!$L$43*(1+Premissas!$B$26),0)</f>
-        <v>1129</v>
-      </c>
-      <c r="E43" s="37" t="n">
-        <f aca="false">Preços!$D$22</f>
-        <v>0.9</v>
-      </c>
-      <c r="F43" s="31" t="n">
-        <f aca="false">C43*E43</f>
-        <v>49.5</v>
-      </c>
-      <c r="G43" s="31" t="n">
-        <f aca="false">D43*E43</f>
-        <v>1016.1</v>
       </c>
     </row>
   </sheetData>
@@ -9508,35 +10266,35 @@
         <v>240</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="C3" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$F$44*(1+Premissas!$B$26),0)</f>
@@ -9561,10 +10319,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C4" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$26),0)</f>
@@ -9589,10 +10347,10 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="C5" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$O$44*(1+Premissas!$B$26),0)</f>
@@ -9617,10 +10375,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C6" s="39" t="n">
         <f aca="false">Estações!$F$44*Premissas!$B$43+Estações!$M$44*Premissas!$B$29+Estações!$O$44*2*Premissas!$B$30</f>
@@ -9645,10 +10403,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="C7" s="39" t="n">
         <f aca="false">(Estações!$F$44+Estações!$M$44)*2+Estações!$O$44*4</f>
@@ -9673,10 +10431,10 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
@@ -9692,10 +10450,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="C9" s="39" t="n">
         <f aca="false">1</f>
@@ -9720,10 +10478,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="C10" s="21" t="n">
         <f aca="false">(C3+C4+C5)*Premissas!$B$44</f>
@@ -9748,10 +10506,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="C11" s="21" t="n">
         <f aca="false">(Estações!$O$44*Premissas!$B$16+Estações!$F$44*Premissas!$B$17+Estações!$M$44*Premissas!$B$19+'A-Interno'!C9*Premissas!$B$20+Estações!$O$44*Premissas!$B$21)*Premissas!$B$22</f>
@@ -9776,10 +10534,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -9795,7 +10553,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -9812,15 +10570,15 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="C16" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$F$44*(1+Premissas!$B$26),0)</f>
@@ -9845,10 +10603,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C17" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$M$44*(1+Premissas!$B$26),0)</f>
@@ -9873,7 +10631,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>155</v>
@@ -9901,7 +10659,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>155</v>
@@ -9929,10 +10687,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C20" s="39" t="n">
         <f aca="false">Estações!$F$44*Premissas!$B$43+Estações!$M$44*Premissas!$B$29+Estações!$O$44*2*Premissas!$B$30</f>
@@ -9957,10 +10715,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="C21" s="39" t="n">
         <f aca="false">(Estações!$F$44+Estações!$M$44)*2+Estações!$O$44*4</f>
@@ -9985,10 +10743,10 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -10004,10 +10762,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="C23" s="21" t="n">
         <f aca="false">(Estações!$O$44*Premissas!$B$16+Estações!$F$44*Premissas!$B$17+Estações!$M$44*Premissas!$B$19+'A-Interno'!C9*Premissas!$B$20+Estações!$O$44*Premissas!$B$21)*Premissas!$B$22</f>
@@ -10032,10 +10790,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
@@ -10051,7 +10809,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
@@ -10068,7 +10826,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
@@ -10103,35 +10861,35 @@
         <v>240</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -10147,10 +10905,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="C4" s="39" t="n">
         <f aca="false">ROUNDUP(Premissas!$B$40*Estações!$O$44/Estações!$O$43,0)</f>
@@ -10175,10 +10933,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="C5" s="21" t="n">
         <f aca="false">C4*30/3600</f>
@@ -10203,15 +10961,15 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="C8" s="39" t="n">
         <f aca="false">ROUNDUP(Estações!$O$44*Premissas!$B$41,0)</f>
@@ -10236,10 +10994,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C9" s="39" t="n">
         <f aca="false">Estações!$O$44</f>
@@ -10264,10 +11022,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="C10" s="21" t="n">
         <f aca="false">C8*1.5</f>
@@ -10292,7 +11050,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -10309,15 +11067,15 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C14" s="39" t="n">
         <f aca="false">Estações!$O$44</f>
@@ -10342,10 +11100,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="C15" s="21" t="n">
         <f aca="false">C14*2</f>
@@ -10370,7 +11128,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
@@ -10387,10 +11145,10 @@
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="C18" s="39" t="n">
         <f aca="false">C8</f>
@@ -10415,7 +11173,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>